<commit_message>
Updated Sunday world cup
</commit_message>
<xml_diff>
--- a/docs/worldcup.xlsx
+++ b/docs/worldcup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rylanpaul/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B6D0D5-8BEF-0744-A445-2947AF29247D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F3F4DC-2D43-3E4A-B6B1-89FC2F43EA69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T" sheetId="1" state="hidden" r:id="rId1"/>
@@ -13305,12 +13305,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -13391,50 +13435,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -38799,13 +38799,13 @@
       <c r="B4" s="145" t="s">
         <v>1798</v>
       </c>
-      <c r="C4" s="146" t="e">
+      <c r="C4" s="146">
         <f>IFERROR(_xlfn.XLOOKUP(B4,Rounds!A$2:A$25,Rounds!B$2:B$25), _xlfn.XLOOKUP(B4,Rounds!D$2:D$25,Rounds!C$2:C$25))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D4" s="146" t="e">
+        <v>1</v>
+      </c>
+      <c r="D4" s="146">
         <f>IFERROR(_xlfn.XLOOKUP(B4,Rounds!A$2:A$25,Rounds!C$2:C$25), _xlfn.XLOOKUP(B4,Rounds!D$2:D$25,Rounds!B$2:B$25))</f>
-        <v>#N/A</v>
+        <v>1</v>
       </c>
       <c r="E4" s="147" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(B4,Rounds!A$2:A$25,Rounds!D$2:D$25), _xlfn.XLOOKUP(B4,Rounds!D$2:D$25,Rounds!A$2:A$25))</f>
@@ -39111,13 +39111,13 @@
       <c r="B7" s="132" t="s">
         <v>1798</v>
       </c>
-      <c r="C7" s="82" t="e">
+      <c r="C7" s="82">
         <f>IFERROR(_xlfn.XLOOKUP(B7,Rounds!A$2:A$25,Rounds!B$2:B$25), _xlfn.XLOOKUP(B7,Rounds!D$2:D$25,Rounds!C$2:C$25))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D7" s="82" t="e">
+        <v>1</v>
+      </c>
+      <c r="D7" s="82">
         <f>IFERROR(_xlfn.XLOOKUP(B7,Rounds!A$2:A$25,Rounds!C$2:C$25), _xlfn.XLOOKUP(B7,Rounds!D$2:D$25,Rounds!B$2:B$25))</f>
-        <v>#N/A</v>
+        <v>1</v>
       </c>
       <c r="E7" s="134" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(B7,Rounds!A$2:A$25,Rounds!D$2:D$25), _xlfn.XLOOKUP(B7,Rounds!D$2:D$25,Rounds!A$2:A$25))</f>
@@ -39215,13 +39215,13 @@
       <c r="B8" s="149" t="s">
         <v>1798</v>
       </c>
-      <c r="C8" s="150" t="e">
+      <c r="C8" s="150">
         <f>IFERROR(_xlfn.XLOOKUP(B8,Rounds!A$2:A$25,Rounds!B$2:B$25), _xlfn.XLOOKUP(B8,Rounds!D$2:D$25,Rounds!C$2:C$25))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D8" s="150" t="e">
+        <v>1</v>
+      </c>
+      <c r="D8" s="150">
         <f>IFERROR(_xlfn.XLOOKUP(B8,Rounds!A$2:A$25,Rounds!C$2:C$25), _xlfn.XLOOKUP(B8,Rounds!D$2:D$25,Rounds!B$2:B$25))</f>
-        <v>#N/A</v>
+        <v>1</v>
       </c>
       <c r="E8" s="151" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(B8,Rounds!A$2:A$25,Rounds!D$2:D$25), _xlfn.XLOOKUP(B8,Rounds!D$2:D$25,Rounds!A$2:A$25))</f>
@@ -39667,11 +39667,11 @@
       <c r="A4" s="132" t="str">
         <v>Canada</v>
       </c>
-      <c r="B4" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C4" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B4" s="81">
+        <v>1</v>
+      </c>
+      <c r="C4" s="81">
+        <v>1</v>
       </c>
       <c r="D4" s="134" t="str">
         <v>Bosnia and Herzegovina</v>
@@ -39753,11 +39753,11 @@
       <c r="A5" s="132" t="str">
         <v>United States</v>
       </c>
-      <c r="B5" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C5" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B5" s="81">
+        <v>4</v>
+      </c>
+      <c r="C5" s="81">
+        <v>1</v>
       </c>
       <c r="D5" s="134" t="str">
         <v>Paraguay</v>
@@ -39839,11 +39839,11 @@
       <c r="A6" s="132" t="str">
         <v>Haiti</v>
       </c>
-      <c r="B6" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C6" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B6" s="81">
+        <v>0</v>
+      </c>
+      <c r="C6" s="81">
+        <v>1</v>
       </c>
       <c r="D6" s="134" t="str">
         <v>Scotland</v>
@@ -39909,11 +39909,11 @@
       <c r="A7" s="132" t="str">
         <v>Australia</v>
       </c>
-      <c r="B7" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C7" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B7" s="81">
+        <v>2</v>
+      </c>
+      <c r="C7" s="81">
+        <v>0</v>
       </c>
       <c r="D7" s="134" t="str">
         <v>Turkey</v>
@@ -39979,11 +39979,11 @@
       <c r="A8" s="132" t="str">
         <v>Brazil</v>
       </c>
-      <c r="B8" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C8" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B8" s="81">
+        <v>1</v>
+      </c>
+      <c r="C8" s="81">
+        <v>1</v>
       </c>
       <c r="D8" s="134" t="str">
         <v>Morocco</v>
@@ -40049,11 +40049,11 @@
       <c r="A9" s="132" t="str">
         <v>Qatar</v>
       </c>
-      <c r="B9" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C9" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B9" s="81">
+        <v>1</v>
+      </c>
+      <c r="C9" s="81">
+        <v>1</v>
       </c>
       <c r="D9" s="134" t="str">
         <v>Switzerland</v>
@@ -40173,11 +40173,11 @@
       <c r="A11" s="132" t="str">
         <v>Germany</v>
       </c>
-      <c r="B11" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C11" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B11" s="81">
+        <v>7</v>
+      </c>
+      <c r="C11" s="81">
+        <v>1</v>
       </c>
       <c r="D11" s="134" t="str">
         <v>Curaçao</v>
@@ -40227,11 +40227,11 @@
       <c r="A12" s="132" t="str">
         <v>Netherlands</v>
       </c>
-      <c r="B12" s="81" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="C12" s="81" t="e">
-        <v>#N/A</v>
+      <c r="B12" s="81">
+        <v>2</v>
+      </c>
+      <c r="C12" s="81">
+        <v>2</v>
       </c>
       <c r="D12" s="134" t="str">
         <v>Japan</v>
@@ -40931,25 +40931,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:95" ht="47" x14ac:dyDescent="0.2">
-      <c r="A1" s="171" t="str" cm="1">
+      <c r="A1" s="182" t="str" cm="1">
         <f t="array" ref="A1">INDEX(T,2,lang)</f>
         <v>2026 World Cup Final Tournament Schedule</v>
       </c>
-      <c r="B1" s="171"/>
-      <c r="C1" s="171"/>
-      <c r="D1" s="171"/>
-      <c r="E1" s="171"/>
-      <c r="F1" s="171"/>
-      <c r="G1" s="171"/>
-      <c r="H1" s="171"/>
-      <c r="I1" s="171"/>
-      <c r="J1" s="171"/>
-      <c r="K1" s="171"/>
-      <c r="L1" s="171"/>
-      <c r="M1" s="171"/>
-      <c r="N1" s="171"/>
-      <c r="O1" s="171"/>
-      <c r="P1" s="171"/>
+      <c r="B1" s="182"/>
+      <c r="C1" s="182"/>
+      <c r="D1" s="182"/>
+      <c r="E1" s="182"/>
+      <c r="F1" s="182"/>
+      <c r="G1" s="182"/>
+      <c r="H1" s="182"/>
+      <c r="I1" s="182"/>
+      <c r="J1" s="182"/>
+      <c r="K1" s="182"/>
+      <c r="L1" s="182"/>
+      <c r="M1" s="182"/>
+      <c r="N1" s="182"/>
+      <c r="O1" s="182"/>
+      <c r="P1" s="182"/>
       <c r="S1" s="123"/>
       <c r="T1" s="123"/>
       <c r="AC1" s="123"/>
@@ -40996,11 +40996,11 @@
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
       <c r="N3" s="10"/>
-      <c r="O3" s="172" t="str">
+      <c r="O3" s="183" t="str">
         <f>"Language: " &amp; Settings!C4</f>
         <v>Language: English</v>
       </c>
-      <c r="P3" s="172"/>
+      <c r="P3" s="183"/>
       <c r="S3" s="123"/>
       <c r="T3" s="123"/>
       <c r="AC3" s="123"/>
@@ -41018,43 +41018,43 @@
     </row>
     <row r="4" spans="1:95" ht="3" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:95" x14ac:dyDescent="0.2">
-      <c r="A5" s="173" t="str" cm="1">
+      <c r="A5" s="184" t="str" cm="1">
         <f t="array" ref="A5">INDEX(T,3,lang)</f>
         <v>Group Stage</v>
       </c>
-      <c r="B5" s="174"/>
-      <c r="C5" s="174"/>
-      <c r="D5" s="174"/>
-      <c r="E5" s="174"/>
-      <c r="F5" s="174"/>
-      <c r="G5" s="174"/>
-      <c r="H5" s="175"/>
-      <c r="J5" s="179" t="s">
+      <c r="B5" s="185"/>
+      <c r="C5" s="185"/>
+      <c r="D5" s="185"/>
+      <c r="E5" s="185"/>
+      <c r="F5" s="185"/>
+      <c r="G5" s="185"/>
+      <c r="H5" s="186"/>
+      <c r="J5" s="190" t="s">
         <v>3166</v>
       </c>
-      <c r="K5" s="180"/>
-      <c r="L5" s="180"/>
-      <c r="M5" s="180"/>
-      <c r="N5" s="180"/>
-      <c r="O5" s="180"/>
-      <c r="P5" s="181"/>
+      <c r="K5" s="191"/>
+      <c r="L5" s="191"/>
+      <c r="M5" s="191"/>
+      <c r="N5" s="191"/>
+      <c r="O5" s="191"/>
+      <c r="P5" s="192"/>
     </row>
     <row r="6" spans="1:95" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="176"/>
-      <c r="B6" s="177"/>
-      <c r="C6" s="177"/>
-      <c r="D6" s="177"/>
-      <c r="E6" s="177"/>
-      <c r="F6" s="177"/>
-      <c r="G6" s="177"/>
-      <c r="H6" s="178"/>
-      <c r="J6" s="182"/>
-      <c r="K6" s="183"/>
-      <c r="L6" s="183"/>
-      <c r="M6" s="183"/>
-      <c r="N6" s="183"/>
-      <c r="O6" s="183"/>
-      <c r="P6" s="184"/>
+      <c r="A6" s="187"/>
+      <c r="B6" s="188"/>
+      <c r="C6" s="188"/>
+      <c r="D6" s="188"/>
+      <c r="E6" s="188"/>
+      <c r="F6" s="188"/>
+      <c r="G6" s="188"/>
+      <c r="H6" s="189"/>
+      <c r="J6" s="193"/>
+      <c r="K6" s="194"/>
+      <c r="L6" s="194"/>
+      <c r="M6" s="194"/>
+      <c r="N6" s="194"/>
+      <c r="O6" s="194"/>
+      <c r="P6" s="195"/>
       <c r="R6" s="123" t="s">
         <v>3167</v>
       </c>
@@ -41164,37 +41164,37 @@
       <c r="BI6" s="128" t="s">
         <v>3178</v>
       </c>
-      <c r="BK6" s="165" t="s">
+      <c r="BK6" s="176" t="s">
         <v>3179</v>
       </c>
-      <c r="BL6" s="166"/>
-      <c r="BM6" s="166"/>
-      <c r="BN6" s="166"/>
-      <c r="BO6" s="167"/>
-      <c r="BR6" s="165" t="str" cm="1">
+      <c r="BL6" s="177"/>
+      <c r="BM6" s="177"/>
+      <c r="BN6" s="177"/>
+      <c r="BO6" s="178"/>
+      <c r="BR6" s="176" t="str" cm="1">
         <f t="array" ref="BR6">INDEX(T,4,lang)</f>
         <v>Round of 16</v>
       </c>
-      <c r="BS6" s="166"/>
-      <c r="BT6" s="166"/>
-      <c r="BU6" s="166"/>
-      <c r="BV6" s="167"/>
-      <c r="BY6" s="165" t="str" cm="1">
+      <c r="BS6" s="177"/>
+      <c r="BT6" s="177"/>
+      <c r="BU6" s="177"/>
+      <c r="BV6" s="178"/>
+      <c r="BY6" s="176" t="str" cm="1">
         <f t="array" ref="BY6">INDEX(T,5,lang)</f>
         <v>Quarterfinals</v>
       </c>
-      <c r="BZ6" s="166"/>
-      <c r="CA6" s="166"/>
-      <c r="CB6" s="166"/>
-      <c r="CC6" s="167"/>
-      <c r="CF6" s="165" t="str" cm="1">
+      <c r="BZ6" s="177"/>
+      <c r="CA6" s="177"/>
+      <c r="CB6" s="177"/>
+      <c r="CC6" s="178"/>
+      <c r="CF6" s="176" t="str" cm="1">
         <f t="array" ref="CF6">INDEX(T,6,lang)</f>
         <v>Semi-Finals</v>
       </c>
-      <c r="CG6" s="166"/>
-      <c r="CH6" s="166"/>
-      <c r="CI6" s="166"/>
-      <c r="CJ6" s="167"/>
+      <c r="CG6" s="177"/>
+      <c r="CH6" s="177"/>
+      <c r="CI6" s="177"/>
+      <c r="CJ6" s="178"/>
     </row>
     <row r="7" spans="1:95" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11">
@@ -41271,26 +41271,26 @@
         <v>1</v>
       </c>
       <c r="AY7" s="126"/>
-      <c r="BK7" s="168"/>
-      <c r="BL7" s="169"/>
-      <c r="BM7" s="169"/>
-      <c r="BN7" s="169"/>
-      <c r="BO7" s="170"/>
-      <c r="BR7" s="168"/>
-      <c r="BS7" s="169"/>
-      <c r="BT7" s="169"/>
-      <c r="BU7" s="169"/>
-      <c r="BV7" s="170"/>
-      <c r="BY7" s="168"/>
-      <c r="BZ7" s="169"/>
-      <c r="CA7" s="169"/>
-      <c r="CB7" s="169"/>
-      <c r="CC7" s="170"/>
-      <c r="CF7" s="168"/>
-      <c r="CG7" s="169"/>
-      <c r="CH7" s="169"/>
-      <c r="CI7" s="169"/>
-      <c r="CJ7" s="170"/>
+      <c r="BK7" s="179"/>
+      <c r="BL7" s="180"/>
+      <c r="BM7" s="180"/>
+      <c r="BN7" s="180"/>
+      <c r="BO7" s="181"/>
+      <c r="BR7" s="179"/>
+      <c r="BS7" s="180"/>
+      <c r="BT7" s="180"/>
+      <c r="BU7" s="180"/>
+      <c r="BV7" s="181"/>
+      <c r="BY7" s="179"/>
+      <c r="BZ7" s="180"/>
+      <c r="CA7" s="180"/>
+      <c r="CB7" s="180"/>
+      <c r="CC7" s="181"/>
+      <c r="CF7" s="179"/>
+      <c r="CG7" s="180"/>
+      <c r="CH7" s="180"/>
+      <c r="CI7" s="180"/>
+      <c r="CJ7" s="181"/>
     </row>
     <row r="8" spans="1:95" x14ac:dyDescent="0.2">
       <c r="A8" s="16">
@@ -41559,8 +41559,12 @@
         <f>AE14</f>
         <v>Canada</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="20"/>
+      <c r="F9" s="19">
+        <v>1</v>
+      </c>
+      <c r="G9" s="20">
+        <v>1</v>
+      </c>
       <c r="H9" s="80" t="str">
         <f>AE15</f>
         <v>Bosnia and Herzegovina</v>
@@ -41599,43 +41603,43 @@
       </c>
       <c r="S9" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Canada_draw</v>
       </c>
       <c r="T9" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Bosnia and Herzegovina_draw</v>
       </c>
       <c r="U9" s="123">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" s="123">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W9" s="123">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X9" s="123">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y9" s="123">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z9" s="123">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA9" s="123">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB9" s="123" t="str">
+      <c r="AB9" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD9" s="123">
         <f>COUNTIF(AR8:AR11,CONCATENATE("&gt;=",AR9))</f>
@@ -41820,8 +41824,12 @@
         <f>AE26</f>
         <v>United States</v>
       </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="20"/>
+      <c r="F10" s="19">
+        <v>4</v>
+      </c>
+      <c r="G10" s="20">
+        <v>1</v>
+      </c>
       <c r="H10" s="80" t="str">
         <f>AE27</f>
         <v>Paraguay</v>
@@ -41860,11 +41868,11 @@
       </c>
       <c r="S10" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>United States_win</v>
       </c>
       <c r="T10" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Paraguay_lose</v>
       </c>
       <c r="U10" s="123">
         <f t="shared" si="8"/>
@@ -41894,9 +41902,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB10" s="123" t="str">
+      <c r="AB10" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AD10" s="123">
         <f>COUNTIF(AR8:AR11,CONCATENATE("&gt;=",AR10))</f>
@@ -42018,7 +42026,7 @@
         <f>BH10/BH12</f>
         <v>0</v>
       </c>
-      <c r="BK10" s="163">
+      <c r="BK10" s="173">
         <v>74</v>
       </c>
       <c r="BL10" s="24" t="str">
@@ -42079,8 +42087,12 @@
         <f>AE22</f>
         <v>Haiti</v>
       </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="20"/>
+      <c r="F11" s="19">
+        <v>0</v>
+      </c>
+      <c r="G11" s="20">
+        <v>1</v>
+      </c>
       <c r="H11" s="80" t="str">
         <f>AE23</f>
         <v>Scotland</v>
@@ -42119,11 +42131,11 @@
       </c>
       <c r="S11" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Haiti_lose</v>
       </c>
       <c r="T11" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Scotland_win</v>
       </c>
       <c r="U11" s="123">
         <f t="shared" si="8"/>
@@ -42153,9 +42165,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB11" s="123" t="str">
+      <c r="AB11" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="AD11" s="123">
         <f>COUNTIF(AR8:AR11,CONCATENATE("&gt;=",AR11))</f>
@@ -42277,7 +42289,7 @@
         <f>BH11/BH12</f>
         <v>0</v>
       </c>
-      <c r="BK11" s="164"/>
+      <c r="BK11" s="174"/>
       <c r="BL11" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!G3,AK80:AS91,9,FALSE),"3rd Group A/B/C/D/F")</f>
         <v>3rd Group A/B/C/D/F</v>
@@ -42342,8 +42354,12 @@
         <f>AE28</f>
         <v>Australia</v>
       </c>
-      <c r="F12" s="19"/>
-      <c r="G12" s="20"/>
+      <c r="F12" s="19">
+        <v>2</v>
+      </c>
+      <c r="G12" s="20">
+        <v>0</v>
+      </c>
       <c r="H12" s="80" t="str">
         <f>AE29</f>
         <v>Turkey</v>
@@ -42382,11 +42398,11 @@
       </c>
       <c r="S12" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Australia_win</v>
       </c>
       <c r="T12" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Turkey_lose</v>
       </c>
       <c r="U12" s="123">
         <f t="shared" si="8"/>
@@ -42416,9 +42432,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB12" s="123" t="str">
+      <c r="AB12" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AF12" s="123">
         <f t="shared" ref="AF12:AH12" si="12">MAX(AF8:AF11)-MIN(AF8:AF11)+1</f>
@@ -42511,7 +42527,7 @@
       <c r="BO12" s="21"/>
       <c r="BP12" s="114"/>
       <c r="BQ12" s="112"/>
-      <c r="BR12" s="163">
+      <c r="BR12" s="173">
         <v>89</v>
       </c>
       <c r="BS12" s="24" t="str">
@@ -42565,8 +42581,12 @@
         <f>AE20</f>
         <v>Brazil</v>
       </c>
-      <c r="F13" s="19"/>
-      <c r="G13" s="20"/>
+      <c r="F13" s="19">
+        <v>1</v>
+      </c>
+      <c r="G13" s="20">
+        <v>1</v>
+      </c>
       <c r="H13" s="80" t="str">
         <f>AE21</f>
         <v>Morocco</v>
@@ -42577,43 +42597,43 @@
       </c>
       <c r="S13" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Brazil_draw</v>
       </c>
       <c r="T13" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Morocco_draw</v>
       </c>
       <c r="U13" s="123">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" s="123">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W13" s="123">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X13" s="123">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y13" s="123">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z13" s="123">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA13" s="123">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB13" s="123" t="str">
+      <c r="AB13" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="BK13" s="21" t="str" cm="1">
         <f t="array" ref="BK13">INDEX(T,24+MONTH(BP13),lang) &amp; " " &amp; DAY(BP13) &amp; ", " &amp; YEAR(BP13) &amp; "   " &amp; (IF(HOUR(BP13)&lt;10,0,"")&amp;HOUR(BP13)) &amp; ":" &amp;  (IF(MINUTE(BP13)&lt;10,0,"")&amp;MINUTE(BP13))</f>
@@ -42628,7 +42648,7 @@
         <v>46203.875</v>
       </c>
       <c r="BQ13" s="115"/>
-      <c r="BR13" s="164"/>
+      <c r="BR13" s="174"/>
       <c r="BS13" s="26" t="str">
         <f>IF(BP14&gt;BP15,BL14,IF(BP14&lt;BP15,BL15,""))</f>
         <v/>
@@ -42680,8 +42700,12 @@
         <f>AE16</f>
         <v>Qatar</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
+      <c r="F14" s="19">
+        <v>1</v>
+      </c>
+      <c r="G14" s="20">
+        <v>1</v>
+      </c>
       <c r="H14" s="80" t="str">
         <f>AE17</f>
         <v>Switzerland</v>
@@ -42720,43 +42744,43 @@
       </c>
       <c r="S14" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Qatar_draw</v>
       </c>
       <c r="T14" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Switzerland_draw</v>
       </c>
       <c r="U14" s="123">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" s="123">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W14" s="123">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X14" s="123">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y14" s="123">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z14" s="123">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA14" s="123">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB14" s="123" t="str">
+      <c r="AB14" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD14" s="123">
         <f>COUNTIF(AR14:AR17,CONCATENATE("&gt;=",AR14))</f>
@@ -42772,7 +42796,7 @@
       </c>
       <c r="AG14" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE14 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH14" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE14 &amp; "_lose")</f>
@@ -42780,11 +42804,11 @@
       </c>
       <c r="AI14" s="123">
         <f>SUMIF($E$7:$E$78,$AE14,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE14,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ14" s="123">
         <f>SUMIF($E$7:$E$78,$AE14,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE14,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL14" s="123">
         <f>AI14-AJ14</f>
@@ -42796,15 +42820,15 @@
       </c>
       <c r="AN14" s="123">
         <f>AF14*3+AG14</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO14" s="123">
         <f>AN14/AN18*10+BA14</f>
-        <v>0</v>
+        <v>5.9901960784313726</v>
       </c>
       <c r="AP14" s="123">
         <f>AO14*10000000+BI14*100+AM14/AM18*10+AI14/AI18*1++IF(AQ14=0,ROW(),AQ14)/2000000</f>
-        <v>7.7824000000000003E-4</v>
+        <v>59902060.304699808</v>
       </c>
       <c r="AQ14" s="126">
         <f>VLOOKUP(AE14,db_fifarank,2,FALSE)</f>
@@ -42812,7 +42836,7 @@
       </c>
       <c r="AR14" s="125">
         <f>AP14/AP18</f>
-        <v>7.7759871434028365E-4</v>
+        <v>0.99999998330530815</v>
       </c>
       <c r="AS14" s="125" t="str">
         <f>IF(SUM(AF14:AH17)=12,J15,"1B")</f>
@@ -42824,15 +42848,15 @@
       </c>
       <c r="AU14" s="126" cm="1">
         <f t="array" ref="AU14">SUMPRODUCT(($S$7:$S$78=AE14&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE14&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV14" s="126" cm="1">
         <f t="array" ref="AV14">SUMPRODUCT(($E$7:$E$78=AE14)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE14)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW14" s="126" cm="1">
         <f t="array" ref="AW14">SUMPRODUCT(($E$7:$E$78=AE14)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE14)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX14" s="126">
         <f>AV14-AW14</f>
@@ -42844,11 +42868,11 @@
       </c>
       <c r="AZ14" s="126">
         <f>AT14/AT18*1000+AU14/AU18*100+AY14/AY18*10+AV14/AV18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BA14" s="126">
         <f>AZ14/AZ18</f>
-        <v>0</v>
+        <v>0.99019607843137258</v>
       </c>
       <c r="BB14" s="126" cm="1">
         <f t="array" ref="BB14">SUMPRODUCT(($S$7:$S$78=AE14&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE14&amp;"_win")*($X$7:$X$78))</f>
@@ -42856,15 +42880,15 @@
       </c>
       <c r="BC14" s="126" cm="1">
         <f t="array" ref="BC14">SUMPRODUCT(($S$7:$S$78=AE14&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE14&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD14" s="126" cm="1">
         <f t="array" ref="BD14">SUMPRODUCT(($E$7:$E$78=AE14)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE14)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE14" s="126" cm="1">
         <f t="array" ref="BE14">SUMPRODUCT(($E$7:$E$78=AE14)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE14)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF14" s="126">
         <f>BD14-BE14</f>
@@ -42876,13 +42900,13 @@
       </c>
       <c r="BH14" s="126">
         <f>BB14/BB18*1000+BC14/BC18*100+BG14/BG18*10+BD14/BD18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BI14" s="126">
         <f>BH14/BH18</f>
-        <v>0</v>
-      </c>
-      <c r="BK14" s="163">
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="BK14" s="173">
         <v>77</v>
       </c>
       <c r="BL14" s="24" t="str">
@@ -42955,7 +42979,7 @@
       </c>
       <c r="K15" s="31">
         <f>L15+M15+N15</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" s="31">
         <f>VLOOKUP(1,AD14:AN17,3,FALSE)</f>
@@ -42963,7 +42987,7 @@
       </c>
       <c r="M15" s="31">
         <f>VLOOKUP(1,AD14:AN17,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" s="31">
         <f>VLOOKUP(1,AD14:AN17,5,FALSE)</f>
@@ -42971,11 +42995,11 @@
       </c>
       <c r="O15" s="31" t="str">
         <f>VLOOKUP(1,AD14:AN17,6,FALSE) &amp; " - " &amp; VLOOKUP(1,AD14:AN17,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P15" s="32">
         <f>L15*3+M15</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" s="123">
         <f>DATE(2026,6,14)+TIME(12,0,0)+gmt_delta</f>
@@ -43035,7 +43059,7 @@
       </c>
       <c r="AG15" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE15 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH15" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE15 &amp; "_lose")</f>
@@ -43043,11 +43067,11 @@
       </c>
       <c r="AI15" s="123">
         <f>SUMIF($E$7:$E$78,$AE15,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE15,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ15" s="123">
         <f>SUMIF($E$7:$E$78,$AE15,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE15,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL15" s="123">
         <f>AI15-AJ15</f>
@@ -43059,15 +43083,15 @@
       </c>
       <c r="AN15" s="123">
         <f>AF15*3+AG15</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO15" s="123">
         <f>AN15/AN18*10+BA15</f>
-        <v>0</v>
+        <v>5.9901960784313726</v>
       </c>
       <c r="AP15" s="123">
         <f>AO15*10000000+BI15*100+AM15/AM18*10+AI15/AI18*1++IF(AQ15=0,ROW(),AQ15)/2000000</f>
-        <v>6.9291999999999997E-4</v>
+        <v>59902060.304614484</v>
       </c>
       <c r="AQ15" s="126">
         <f>VLOOKUP(AE15,db_fifarank,2,FALSE)</f>
@@ -43075,7 +43099,7 @@
       </c>
       <c r="AR15" s="125">
         <f>AP15/AP18</f>
-        <v>6.9234901976340118E-4</v>
+        <v>0.99999998330388373</v>
       </c>
       <c r="AS15" s="125" t="str">
         <f>IF(SUM(AF14:AH17)=12,J16,"2B")</f>
@@ -43087,15 +43111,15 @@
       </c>
       <c r="AU15" s="126" cm="1">
         <f t="array" ref="AU15">SUMPRODUCT(($S$7:$S$78=AE15&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE15&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV15" s="126" cm="1">
         <f t="array" ref="AV15">SUMPRODUCT(($E$7:$E$78=AE15)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE15)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW15" s="126" cm="1">
         <f t="array" ref="AW15">SUMPRODUCT(($E$7:$E$78=AE15)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE15)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX15" s="126">
         <f>AV15-AW15</f>
@@ -43107,11 +43131,11 @@
       </c>
       <c r="AZ15" s="126">
         <f>AT15/AT18*1000+AU15/AU18*100+AY15/AY18*10+AV15/AV18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BA15" s="126">
         <f>AZ15/AZ18</f>
-        <v>0</v>
+        <v>0.99019607843137258</v>
       </c>
       <c r="BB15" s="126" cm="1">
         <f t="array" ref="BB15">SUMPRODUCT(($S$7:$S$78=AE15&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE15&amp;"_win")*($X$7:$X$78))</f>
@@ -43119,15 +43143,15 @@
       </c>
       <c r="BC15" s="126" cm="1">
         <f t="array" ref="BC15">SUMPRODUCT(($S$7:$S$78=AE15&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE15&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD15" s="126" cm="1">
         <f t="array" ref="BD15">SUMPRODUCT(($E$7:$E$78=AE15)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE15)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE15" s="126" cm="1">
         <f t="array" ref="BE15">SUMPRODUCT(($E$7:$E$78=AE15)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE15)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF15" s="126">
         <f>BD15-BE15</f>
@@ -43139,13 +43163,13 @@
       </c>
       <c r="BH15" s="126">
         <f>BB15/BB18*1000+BC15/BC18*100+BG15/BG18*10+BD15/BD18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BI15" s="126">
         <f>BH15/BH18</f>
-        <v>0</v>
-      </c>
-      <c r="BK15" s="164"/>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="BK15" s="174"/>
       <c r="BL15" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!I3,AK80:AS91,9,FALSE),"3rd Group C/D/F/G/H")</f>
         <v>3rd Group C/D/F/G/H</v>
@@ -43203,8 +43227,12 @@
         <f>AE32</f>
         <v>Germany</v>
       </c>
-      <c r="F16" s="19"/>
-      <c r="G16" s="20"/>
+      <c r="F16" s="19">
+        <v>7</v>
+      </c>
+      <c r="G16" s="20">
+        <v>1</v>
+      </c>
       <c r="H16" s="80" t="str">
         <f>AE33</f>
         <v>Curaçao</v>
@@ -43215,7 +43243,7 @@
       </c>
       <c r="K16" s="23">
         <f>L16+M16+N16</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" s="23">
         <f>VLOOKUP(2,AD14:AN17,3,FALSE)</f>
@@ -43223,7 +43251,7 @@
       </c>
       <c r="M16" s="23">
         <f>VLOOKUP(2,AD14:AN17,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="23">
         <f>VLOOKUP(2,AD14:AN17,5,FALSE)</f>
@@ -43231,11 +43259,11 @@
       </c>
       <c r="O16" s="23" t="str">
         <f>VLOOKUP(2,AD14:AN17,6,FALSE) &amp; " - " &amp; VLOOKUP(2,AD14:AN17,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P16" s="34">
         <f>L16*3+M16</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R16" s="123">
         <f>DATE(2026,6,14)+TIME(6,0,0)+gmt_delta</f>
@@ -43243,11 +43271,11 @@
       </c>
       <c r="S16" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Germany_win</v>
       </c>
       <c r="T16" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Curaçao_lose</v>
       </c>
       <c r="U16" s="123">
         <f t="shared" si="8"/>
@@ -43277,9 +43305,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB16" s="123" t="str">
+      <c r="AB16" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AD16" s="123">
         <f>COUNTIF(AR14:AR17,CONCATENATE("&gt;=",AR16))</f>
@@ -43295,7 +43323,7 @@
       </c>
       <c r="AG16" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE16 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH16" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE16 &amp; "_lose")</f>
@@ -43303,11 +43331,11 @@
       </c>
       <c r="AI16" s="123">
         <f>SUMIF($E$7:$E$78,$AE16,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE16,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ16" s="123">
         <f>SUMIF($E$7:$E$78,$AE16,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE16,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL16" s="123">
         <f>AI16-AJ16</f>
@@ -43319,15 +43347,15 @@
       </c>
       <c r="AN16" s="123">
         <f>AF16*3+AG16</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO16" s="123">
         <f>AN16/AN18*10+BA16</f>
-        <v>0</v>
+        <v>5.9901960784313726</v>
       </c>
       <c r="AP16" s="123">
         <f>AO16*10000000+BI16*100+AM16/AM18*10+AI16/AI18*1++IF(AQ16=0,ROW(),AQ16)/2000000</f>
-        <v>7.2747999999999997E-4</v>
+        <v>59902060.304649048</v>
       </c>
       <c r="AQ16" s="126">
         <f>VLOOKUP(AE16,db_fifarank,2,FALSE)</f>
@@ -43335,7 +43363,7 @@
       </c>
       <c r="AR16" s="125">
         <f>AP16/AP18</f>
-        <v>7.268805416173282E-4</v>
+        <v>0.99999998330446072</v>
       </c>
       <c r="AT16" s="126" cm="1">
         <f t="array" ref="AT16">SUMPRODUCT(($S$7:$S$78=AE16&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE16&amp;"_win")*($U$7:$U$78))</f>
@@ -43343,15 +43371,15 @@
       </c>
       <c r="AU16" s="126" cm="1">
         <f t="array" ref="AU16">SUMPRODUCT(($S$7:$S$78=AE16&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE16&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV16" s="126" cm="1">
         <f t="array" ref="AV16">SUMPRODUCT(($E$7:$E$78=AE16)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE16)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW16" s="126" cm="1">
         <f t="array" ref="AW16">SUMPRODUCT(($E$7:$E$78=AE16)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE16)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX16" s="126">
         <f>AV16-AW16</f>
@@ -43363,11 +43391,11 @@
       </c>
       <c r="AZ16" s="126">
         <f>AT16/AT18*1000+AU16/AU18*100+AY16/AY18*10+AV16/AV18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BA16" s="126">
         <f>AZ16/AZ18</f>
-        <v>0</v>
+        <v>0.99019607843137258</v>
       </c>
       <c r="BB16" s="126" cm="1">
         <f t="array" ref="BB16">SUMPRODUCT(($S$7:$S$78=AE16&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE16&amp;"_win")*($X$7:$X$78))</f>
@@ -43375,15 +43403,15 @@
       </c>
       <c r="BC16" s="126" cm="1">
         <f t="array" ref="BC16">SUMPRODUCT(($S$7:$S$78=AE16&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE16&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD16" s="126" cm="1">
         <f t="array" ref="BD16">SUMPRODUCT(($E$7:$E$78=AE16)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE16)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE16" s="126" cm="1">
         <f t="array" ref="BE16">SUMPRODUCT(($E$7:$E$78=AE16)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE16)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF16" s="126">
         <f>BD16-BE16</f>
@@ -43395,11 +43423,11 @@
       </c>
       <c r="BH16" s="126">
         <f>BB16/BB18*1000+BC16/BC18*100+BG16/BG18*10+BD16/BD18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BI16" s="126">
         <f>BH16/BH18</f>
-        <v>0</v>
+        <v>0.99019607843137258</v>
       </c>
       <c r="BK16" s="21"/>
       <c r="BL16" s="21"/>
@@ -43415,7 +43443,7 @@
       <c r="BV16" s="21"/>
       <c r="BW16" s="114"/>
       <c r="BX16" s="112"/>
-      <c r="BY16" s="163">
+      <c r="BY16" s="173">
         <v>97</v>
       </c>
       <c r="BZ16" s="24" t="str">
@@ -43455,8 +43483,12 @@
         <f>AE38</f>
         <v>Netherlands</v>
       </c>
-      <c r="F17" s="19"/>
-      <c r="G17" s="20"/>
+      <c r="F17" s="19">
+        <v>2</v>
+      </c>
+      <c r="G17" s="20">
+        <v>2</v>
+      </c>
       <c r="H17" s="80" t="str">
         <f>AE39</f>
         <v>Japan</v>
@@ -43467,7 +43499,7 @@
       </c>
       <c r="K17" s="23">
         <f>L17+M17+N17</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" s="23">
         <f>VLOOKUP(3,AD14:AN17,3,FALSE)</f>
@@ -43475,7 +43507,7 @@
       </c>
       <c r="M17" s="23">
         <f>VLOOKUP(3,AD14:AN17,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17" s="23">
         <f>VLOOKUP(3,AD14:AN17,5,FALSE)</f>
@@ -43483,11 +43515,11 @@
       </c>
       <c r="O17" s="23" t="str">
         <f>VLOOKUP(3,AD14:AN17,6,FALSE) &amp; " - " &amp; VLOOKUP(3,AD14:AN17,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P17" s="34">
         <f>L17*3+M17</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17" s="123">
         <f>DATE(2026,6,14)+TIME(9,0,0)+gmt_delta</f>
@@ -43495,43 +43527,43 @@
       </c>
       <c r="S17" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Netherlands_draw</v>
       </c>
       <c r="T17" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Japan_draw</v>
       </c>
       <c r="U17" s="123">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V17" s="123">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W17" s="123">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X17" s="123">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y17" s="123">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z17" s="123">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AA17" s="123">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB17" s="123" t="str">
+      <c r="AB17" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD17" s="123">
         <f>COUNTIF(AR14:AR17,CONCATENATE("&gt;=",AR17))</f>
@@ -43547,7 +43579,7 @@
       </c>
       <c r="AG17" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE17 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH17" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE17 &amp; "_lose")</f>
@@ -43555,11 +43587,11 @@
       </c>
       <c r="AI17" s="123">
         <f>SUMIF($E$7:$E$78,$AE17,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE17,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ17" s="123">
         <f>SUMIF($E$7:$E$78,$AE17,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE17,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL17" s="123">
         <f>AI17-AJ17</f>
@@ -43571,15 +43603,15 @@
       </c>
       <c r="AN17" s="123">
         <f>AF17*3+AG17</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO17" s="123">
         <f>AN17/AN18*10+BA17</f>
-        <v>0</v>
+        <v>5.9901960784313726</v>
       </c>
       <c r="AP17" s="123">
         <f>AO17*10000000+BI17*100+AM17/AM18*10+AI17/AI18*1++IF(AQ17=0,ROW(),AQ17)/2000000</f>
-        <v>8.2470000000000004E-4</v>
+        <v>59902060.304746263</v>
       </c>
       <c r="AQ17" s="126">
         <f>VLOOKUP(AE17,db_fifarank,2,FALSE)</f>
@@ -43587,7 +43619,7 @@
       </c>
       <c r="AR17" s="125">
         <f>AP17/AP18</f>
-        <v>8.2402043035108958E-4</v>
+        <v>0.99999998330608364</v>
       </c>
       <c r="AT17" s="126" cm="1">
         <f t="array" ref="AT17">SUMPRODUCT(($S$7:$S$78=AE17&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE17&amp;"_win")*($U$7:$U$78))</f>
@@ -43595,15 +43627,15 @@
       </c>
       <c r="AU17" s="126" cm="1">
         <f t="array" ref="AU17">SUMPRODUCT(($S$7:$S$78=AE17&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE17&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV17" s="126" cm="1">
         <f t="array" ref="AV17">SUMPRODUCT(($E$7:$E$78=AE17)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE17)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW17" s="126" cm="1">
         <f t="array" ref="AW17">SUMPRODUCT(($E$7:$E$78=AE17)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE17)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX17" s="126">
         <f>AV17-AW17</f>
@@ -43615,11 +43647,11 @@
       </c>
       <c r="AZ17" s="126">
         <f>AT17/AT18*1000+AU17/AU18*100+AY17/AY18*10+AV17/AV18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BA17" s="126">
         <f>AZ17/AZ18</f>
-        <v>0</v>
+        <v>0.99019607843137258</v>
       </c>
       <c r="BB17" s="126" cm="1">
         <f t="array" ref="BB17">SUMPRODUCT(($S$7:$S$78=AE17&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE17&amp;"_win")*($X$7:$X$78))</f>
@@ -43627,15 +43659,15 @@
       </c>
       <c r="BC17" s="126" cm="1">
         <f t="array" ref="BC17">SUMPRODUCT(($S$7:$S$78=AE17&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE17&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD17" s="126" cm="1">
         <f t="array" ref="BD17">SUMPRODUCT(($E$7:$E$78=AE17)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE17)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE17" s="126" cm="1">
         <f t="array" ref="BE17">SUMPRODUCT(($E$7:$E$78=AE17)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE17)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF17" s="126">
         <f>BD17-BE17</f>
@@ -43647,11 +43679,11 @@
       </c>
       <c r="BH17" s="126">
         <f>BB17/BB18*1000+BC17/BC18*100+BG17/BG18*10+BD17/BD18</f>
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="BI17" s="126">
         <f>BH17/BH18</f>
-        <v>0</v>
+        <v>0.99019607843137258</v>
       </c>
       <c r="BK17" s="21" t="str" cm="1">
         <f t="array" ref="BK17">INDEX(T,24+MONTH(BP17),lang) &amp; " " &amp; DAY(BP17) &amp; ", " &amp; YEAR(BP17) &amp; "   " &amp; (IF(HOUR(BP17)&lt;10,0,"")&amp;HOUR(BP17)) &amp; ":" &amp;  (IF(MINUTE(BP17)&lt;10,0,"")&amp;MINUTE(BP17))</f>
@@ -43673,7 +43705,7 @@
       <c r="BV17" s="21"/>
       <c r="BW17" s="114"/>
       <c r="BX17" s="115"/>
-      <c r="BY17" s="164"/>
+      <c r="BY17" s="174"/>
       <c r="BZ17" s="26" t="str">
         <f>IF(BW20&gt;BW21,BS20,IF(BW20&lt;BW21,BS21,""))</f>
         <v/>
@@ -43723,7 +43755,7 @@
       </c>
       <c r="K18" s="36">
         <f>L18+M18+N18</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" s="36">
         <f>VLOOKUP(4,AD14:AN17,3,FALSE)</f>
@@ -43731,7 +43763,7 @@
       </c>
       <c r="M18" s="36">
         <f>VLOOKUP(4,AD14:AN17,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="36">
         <f>VLOOKUP(4,AD14:AN17,5,FALSE)</f>
@@ -43739,11 +43771,11 @@
       </c>
       <c r="O18" s="36" t="str">
         <f>VLOOKUP(4,AD14:AN17,6,FALSE) &amp; " - " &amp; VLOOKUP(4,AD14:AN17,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P18" s="37">
         <f>L18*3+M18</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R18" s="123">
         <f>DATE(2026,6,14)+TIME(15,0,0)+gmt_delta</f>
@@ -43803,7 +43835,7 @@
       </c>
       <c r="AI18" s="123">
         <f>MAX(AI14:AI17)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL18" s="123">
         <f>MIN(AL14:AL17)</f>
@@ -43815,15 +43847,15 @@
       </c>
       <c r="AN18" s="123">
         <f>MAX(AN14:AN17)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO18" s="123">
         <f>MAX(AO14:AO17)+1</f>
-        <v>1</v>
+        <v>6.9901960784313726</v>
       </c>
       <c r="AP18" s="123">
         <f>MAX(AP14:AP17)+1</f>
-        <v>1.0008246999999999</v>
+        <v>59902061.304746263</v>
       </c>
       <c r="AT18" s="126">
         <f>MAX(AT14:AT17)-MIN(AT14:AT17)+1</f>
@@ -43847,7 +43879,7 @@
       </c>
       <c r="AZ18" s="126">
         <f>MAX(AZ14:AZ17)+1</f>
-        <v>1</v>
+        <v>102</v>
       </c>
       <c r="BB18" s="126">
         <f>MAX(BB14:BB17)-MIN(BB14:BB17)+1</f>
@@ -43871,9 +43903,9 @@
       </c>
       <c r="BH18" s="126">
         <f>MAX(BH14:BH17)+1</f>
-        <v>1</v>
-      </c>
-      <c r="BK18" s="163">
+        <v>102</v>
+      </c>
+      <c r="BK18" s="173">
         <v>73</v>
       </c>
       <c r="BL18" s="24" t="str">
@@ -43977,7 +44009,7 @@
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="BK19" s="164"/>
+      <c r="BK19" s="174"/>
       <c r="BL19" s="26" t="str">
         <f>AS15</f>
         <v>2B</v>
@@ -44122,7 +44154,7 @@
       </c>
       <c r="AD20" s="123">
         <f>COUNTIF(AR20:AR23,CONCATENATE("&gt;=",AR20))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE20" s="124" t="str">
         <f>VLOOKUP("Brazil",T,lang,FALSE)</f>
@@ -44134,7 +44166,7 @@
       </c>
       <c r="AG20" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE20 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH20" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE20 &amp; "_lose")</f>
@@ -44142,11 +44174,11 @@
       </c>
       <c r="AI20" s="123">
         <f>SUMIF($E$7:$E$78,$AE20,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE20,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ20" s="123">
         <f>SUMIF($E$7:$E$78,$AE20,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE20,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL20" s="123">
         <f>AI20-AJ20</f>
@@ -44154,19 +44186,19 @@
       </c>
       <c r="AM20" s="123">
         <f>AL20-AL24</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN20" s="123">
         <f>AF20*3+AG20</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO20" s="123">
         <f>AN20/AN24*10+BA20</f>
-        <v>0</v>
+        <v>3.4805825242718447</v>
       </c>
       <c r="AP20" s="123">
         <f>AO20*10000000+BI20*100+AM20/AM24*10+AI20/AI24*1++IF(AQ20=0,ROW(),AQ20)/2000000</f>
-        <v>8.8058000000000006E-4</v>
+        <v>34805927.13518478</v>
       </c>
       <c r="AQ20" s="126">
         <f>VLOOKUP(AE20,db_fifarank,2,FALSE)</f>
@@ -44174,7 +44206,7 @@
       </c>
       <c r="AR20" s="125">
         <f>AP20/AP24</f>
-        <v>8.7980526108319542E-4</v>
+        <v>0.46407897793145042</v>
       </c>
       <c r="AS20" s="125" t="str">
         <f>IF(SUM(AF20:AH23)=12,J21,"1C")</f>
@@ -44186,15 +44218,15 @@
       </c>
       <c r="AU20" s="126" cm="1">
         <f t="array" ref="AU20">SUMPRODUCT(($S$7:$S$78=AE20&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE20&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV20" s="126" cm="1">
         <f t="array" ref="AV20">SUMPRODUCT(($E$7:$E$78=AE20)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE20)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW20" s="126" cm="1">
         <f t="array" ref="AW20">SUMPRODUCT(($E$7:$E$78=AE20)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE20)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX20" s="126">
         <f>AV20-AW20</f>
@@ -44206,11 +44238,11 @@
       </c>
       <c r="AZ20" s="126">
         <f>AT20/AT24*1000+AU20/AU24*100+AY20/AY24*10+AV20/AV24</f>
-        <v>0</v>
+        <v>50.5</v>
       </c>
       <c r="BA20" s="126">
         <f>AZ20/AZ24</f>
-        <v>0</v>
+        <v>0.98058252427184467</v>
       </c>
       <c r="BB20" s="126" cm="1">
         <f t="array" ref="BB20">SUMPRODUCT(($S$7:$S$78=AE20&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE20&amp;"_win")*($X$7:$X$78))</f>
@@ -44218,15 +44250,15 @@
       </c>
       <c r="BC20" s="126" cm="1">
         <f t="array" ref="BC20">SUMPRODUCT(($S$7:$S$78=AE20&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE20&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD20" s="126" cm="1">
         <f t="array" ref="BD20">SUMPRODUCT(($E$7:$E$78=AE20)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE20)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE20" s="126" cm="1">
         <f t="array" ref="BE20">SUMPRODUCT(($E$7:$E$78=AE20)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE20)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF20" s="126">
         <f>BD20-BE20</f>
@@ -44238,11 +44270,11 @@
       </c>
       <c r="BH20" s="126">
         <f>BB20/BB24*1000+BC20/BC24*100+BG20/BG24*10+BD20/BD24</f>
-        <v>0</v>
+        <v>50.5</v>
       </c>
       <c r="BI20" s="126">
         <f>BH20/BH24</f>
-        <v>0</v>
+        <v>0.98058252427184467</v>
       </c>
       <c r="BK20" s="21"/>
       <c r="BL20" s="21"/>
@@ -44251,7 +44283,7 @@
       <c r="BO20" s="21"/>
       <c r="BP20" s="114"/>
       <c r="BQ20" s="112"/>
-      <c r="BR20" s="163">
+      <c r="BR20" s="173">
         <v>90</v>
       </c>
       <c r="BS20" s="24" t="str">
@@ -44313,15 +44345,15 @@
       </c>
       <c r="J21" s="30" t="str">
         <f>VLOOKUP(1,AD20:AN23,2,FALSE)</f>
-        <v>Brazil</v>
+        <v>Scotland</v>
       </c>
       <c r="K21" s="31">
         <f>L21+M21+N21</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="31">
         <f>VLOOKUP(1,AD20:AN23,3,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" s="31">
         <f>VLOOKUP(1,AD20:AN23,4,FALSE)</f>
@@ -44333,11 +44365,11 @@
       </c>
       <c r="O21" s="31" t="str">
         <f>VLOOKUP(1,AD20:AN23,6,FALSE) &amp; " - " &amp; VLOOKUP(1,AD20:AN23,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 0</v>
       </c>
       <c r="P21" s="32">
         <f>L21*3+M21</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R21" s="123">
         <f>DATE(2026,6,15)+TIME(14,0,0)+gmt_delta</f>
@@ -44385,7 +44417,7 @@
       </c>
       <c r="AD21" s="123">
         <f>COUNTIF(AR20:AR23,CONCATENATE("&gt;=",AR21))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE21" s="124" t="str">
         <f>VLOOKUP("Morocco",T,lang,FALSE)</f>
@@ -44397,7 +44429,7 @@
       </c>
       <c r="AG21" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE21 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH21" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE21 &amp; "_lose")</f>
@@ -44405,11 +44437,11 @@
       </c>
       <c r="AI21" s="123">
         <f>SUMIF($E$7:$E$78,$AE21,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE21,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ21" s="123">
         <f>SUMIF($E$7:$E$78,$AE21,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE21,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL21" s="123">
         <f>AI21-AJ21</f>
@@ -44417,19 +44449,19 @@
       </c>
       <c r="AM21" s="123">
         <f>AL21-AL24</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN21" s="123">
         <f>AF21*3+AG21</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO21" s="123">
         <f>AN21/AN24*10+BA21</f>
-        <v>0</v>
+        <v>3.4805825242718447</v>
       </c>
       <c r="AP21" s="123">
         <f>AO21*10000000+BI21*100+AM21/AM24*10+AI21/AI24*1++IF(AQ21=0,ROW(),AQ21)/2000000</f>
-        <v>8.7793499999999994E-4</v>
+        <v>34805927.135182135</v>
       </c>
       <c r="AQ21" s="126">
         <f>VLOOKUP(AE21,db_fifarank,2,FALSE)</f>
@@ -44437,7 +44469,7 @@
       </c>
       <c r="AR21" s="125">
         <f>AP21/AP24</f>
-        <v>8.771625881681108E-4</v>
+        <v>0.46407897793141517</v>
       </c>
       <c r="AS21" s="125" t="str">
         <f>IF(SUM(AF20:AH23)=12,J22,"2C")</f>
@@ -44449,15 +44481,15 @@
       </c>
       <c r="AU21" s="126" cm="1">
         <f t="array" ref="AU21">SUMPRODUCT(($S$7:$S$78=AE21&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE21&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV21" s="126" cm="1">
         <f t="array" ref="AV21">SUMPRODUCT(($E$7:$E$78=AE21)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE21)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW21" s="126" cm="1">
         <f t="array" ref="AW21">SUMPRODUCT(($E$7:$E$78=AE21)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE21)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX21" s="126">
         <f>AV21-AW21</f>
@@ -44469,11 +44501,11 @@
       </c>
       <c r="AZ21" s="126">
         <f>AT21/AT24*1000+AU21/AU24*100+AY21/AY24*10+AV21/AV24</f>
-        <v>0</v>
+        <v>50.5</v>
       </c>
       <c r="BA21" s="126">
         <f>AZ21/AZ24</f>
-        <v>0</v>
+        <v>0.98058252427184467</v>
       </c>
       <c r="BB21" s="126" cm="1">
         <f t="array" ref="BB21">SUMPRODUCT(($S$7:$S$78=AE21&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE21&amp;"_win")*($X$7:$X$78))</f>
@@ -44481,15 +44513,15 @@
       </c>
       <c r="BC21" s="126" cm="1">
         <f t="array" ref="BC21">SUMPRODUCT(($S$7:$S$78=AE21&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE21&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD21" s="126" cm="1">
         <f t="array" ref="BD21">SUMPRODUCT(($E$7:$E$78=AE21)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE21)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE21" s="126" cm="1">
         <f t="array" ref="BE21">SUMPRODUCT(($E$7:$E$78=AE21)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE21)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF21" s="126">
         <f>BD21-BE21</f>
@@ -44501,11 +44533,11 @@
       </c>
       <c r="BH21" s="126">
         <f>BB21/BB24*1000+BC21/BC24*100+BG21/BG24*10+BD21/BD24</f>
-        <v>0</v>
+        <v>50.5</v>
       </c>
       <c r="BI21" s="126">
         <f>BH21/BH24</f>
-        <v>0</v>
+        <v>0.98058252427184467</v>
       </c>
       <c r="BK21" s="21" t="str" cm="1">
         <f t="array" ref="BK21">INDEX(T,24+MONTH(BP21),lang) &amp; " " &amp; DAY(BP21) &amp; ", " &amp; YEAR(BP21) &amp; "   " &amp; (IF(HOUR(BP21)&lt;10,0,"")&amp;HOUR(BP21)) &amp; ":" &amp;  (IF(MINUTE(BP21)&lt;10,0,"")&amp;MINUTE(BP21))</f>
@@ -44520,7 +44552,7 @@
         <v>46203.041666666672</v>
       </c>
       <c r="BQ21" s="115"/>
-      <c r="BR21" s="164"/>
+      <c r="BR21" s="174"/>
       <c r="BS21" s="26" t="str">
         <f>IF(BP22&gt;BP23,BL22,IF(BP22&lt;BP23,BL23,""))</f>
         <v/>
@@ -44580,11 +44612,11 @@
       </c>
       <c r="J22" s="33" t="str">
         <f>VLOOKUP(2,AD20:AN23,2,FALSE)</f>
-        <v>Morocco</v>
+        <v>Brazil</v>
       </c>
       <c r="K22" s="23">
         <f>L22+M22+N22</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" s="23">
         <f>VLOOKUP(2,AD20:AN23,3,FALSE)</f>
@@ -44592,7 +44624,7 @@
       </c>
       <c r="M22" s="23">
         <f>VLOOKUP(2,AD20:AN23,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="23">
         <f>VLOOKUP(2,AD20:AN23,5,FALSE)</f>
@@ -44600,11 +44632,11 @@
       </c>
       <c r="O22" s="23" t="str">
         <f>VLOOKUP(2,AD20:AN23,6,FALSE) &amp; " - " &amp; VLOOKUP(2,AD20:AN23,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P22" s="34">
         <f>L22*3+M22</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" s="123">
         <f>DATE(2026,6,15)+TIME(8,0,0)+gmt_delta</f>
@@ -44668,7 +44700,7 @@
       </c>
       <c r="AH22" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE22 &amp; "_lose")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI22" s="123">
         <f>SUMIF($E$7:$E$78,$AE22,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE22,$G$7:$G$78)</f>
@@ -44676,11 +44708,11 @@
       </c>
       <c r="AJ22" s="123">
         <f>SUMIF($E$7:$E$78,$AE22,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE22,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL22" s="123">
         <f>AI22-AJ22</f>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM22" s="123">
         <f>AL22-AL24</f>
@@ -44704,7 +44736,7 @@
       </c>
       <c r="AR22" s="125">
         <f>AP22/AP24</f>
-        <v>6.4528677337310309E-4</v>
+        <v>8.6113990622283044E-12</v>
       </c>
       <c r="AT22" s="126" cm="1">
         <f t="array" ref="AT22">SUMPRODUCT(($S$7:$S$78=AE22&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE22&amp;"_win")*($U$7:$U$78))</f>
@@ -44770,7 +44802,7 @@
         <f>BH22/BH24</f>
         <v>0</v>
       </c>
-      <c r="BK22" s="163">
+      <c r="BK22" s="173">
         <v>75</v>
       </c>
       <c r="BL22" s="24" t="str">
@@ -44840,11 +44872,11 @@
       </c>
       <c r="J23" s="33" t="str">
         <f>VLOOKUP(3,AD20:AN23,2,FALSE)</f>
-        <v>Scotland</v>
+        <v>Morocco</v>
       </c>
       <c r="K23" s="23">
         <f>L23+M23+N23</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" s="23">
         <f>VLOOKUP(3,AD20:AN23,3,FALSE)</f>
@@ -44852,7 +44884,7 @@
       </c>
       <c r="M23" s="23">
         <f>VLOOKUP(3,AD20:AN23,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" s="23">
         <f>VLOOKUP(3,AD20:AN23,5,FALSE)</f>
@@ -44860,11 +44892,11 @@
       </c>
       <c r="O23" s="23" t="str">
         <f>VLOOKUP(3,AD20:AN23,6,FALSE) &amp; " - " &amp; VLOOKUP(3,AD20:AN23,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P23" s="34">
         <f>L23*3+M23</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23" s="123">
         <f>DATE(2026,6,16)+TIME(8,0,0)+gmt_delta</f>
@@ -44912,7 +44944,7 @@
       </c>
       <c r="AD23" s="123">
         <f>COUNTIF(AR20:AR23,CONCATENATE("&gt;=",AR23))</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE23" s="124" t="str">
         <f>VLOOKUP("Scotland",T,lang,FALSE)</f>
@@ -44920,7 +44952,7 @@
       </c>
       <c r="AF23" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE23 &amp; "_win")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG23" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE23 &amp; "_draw")</f>
@@ -44932,7 +44964,7 @@
       </c>
       <c r="AI23" s="123">
         <f>SUMIF($E$7:$E$78,$AE23,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE23,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ23" s="123">
         <f>SUMIF($E$7:$E$78,$AE23,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE23,$F$7:$F$78)</f>
@@ -44940,23 +44972,23 @@
       </c>
       <c r="AL23" s="123">
         <f>AI23-AJ23</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM23" s="123">
         <f>AL23-AL24</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AN23" s="123">
         <f>AF23*3+AG23</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO23" s="123">
         <f>AN23/AN24*10+BA23</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="AP23" s="123">
         <f>AO23*10000000+BI23*100+AM23/AM24*10+AI23/AI24*1++IF(AQ23=0,ROW(),AQ23)/2000000</f>
-        <v>7.4917499999999993E-4</v>
+        <v>75000007.167415842</v>
       </c>
       <c r="AQ23" s="126">
         <f>VLOOKUP(AE23,db_fifarank,2,FALSE)</f>
@@ -44964,7 +44996,7 @@
       </c>
       <c r="AR23" s="125">
         <f>AP23/AP24</f>
-        <v>7.4851587189352792E-4</v>
+        <v>0.99999998666666812</v>
       </c>
       <c r="AT23" s="126" cm="1">
         <f t="array" ref="AT23">SUMPRODUCT(($S$7:$S$78=AE23&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE23&amp;"_win")*($U$7:$U$78))</f>
@@ -45030,7 +45062,7 @@
         <f>BH23/BH24</f>
         <v>0</v>
       </c>
-      <c r="BK23" s="164"/>
+      <c r="BK23" s="174"/>
       <c r="BL23" s="26" t="str">
         <f>AS21</f>
         <v>2C</v>
@@ -45057,7 +45089,7 @@
       <c r="CC23" s="21"/>
       <c r="CD23" s="114"/>
       <c r="CE23" s="112"/>
-      <c r="CF23" s="163">
+      <c r="CF23" s="173">
         <v>101</v>
       </c>
       <c r="CG23" s="24" t="str">
@@ -45104,7 +45136,7 @@
       </c>
       <c r="K24" s="36">
         <f>L24+M24+N24</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="36">
         <f>VLOOKUP(4,AD20:AN23,3,FALSE)</f>
@@ -45116,11 +45148,11 @@
       </c>
       <c r="N24" s="36">
         <f>VLOOKUP(4,AD20:AN23,5,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O24" s="36" t="str">
         <f>VLOOKUP(4,AD20:AN23,6,FALSE) &amp; " - " &amp; VLOOKUP(4,AD20:AN23,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>0 - 1</v>
       </c>
       <c r="P24" s="37">
         <f>L24*3+M24</f>
@@ -45172,39 +45204,39 @@
       </c>
       <c r="AF24" s="123">
         <f t="shared" ref="AF24:AH24" si="14">MAX(AF20:AF23)-MIN(AF20:AF23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG24" s="123">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH24" s="123">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI24" s="123">
         <f>MAX(AI20:AI23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL24" s="123">
         <f>MIN(AL20:AL23)</f>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM24" s="123">
         <f>MAX(AM20:AM23)+1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AN24" s="123">
         <f>MAX(AN20:AN23)+1</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AO24" s="123">
         <f>MAX(AO20:AO23)+1</f>
-        <v>1</v>
+        <v>8.5</v>
       </c>
       <c r="AP24" s="123">
         <f>MAX(AP20:AP23)+1</f>
-        <v>1.00088058</v>
+        <v>75000008.167415842</v>
       </c>
       <c r="AT24" s="126">
         <f>MAX(AT20:AT23)-MIN(AT20:AT23)+1</f>
@@ -45212,15 +45244,15 @@
       </c>
       <c r="AU24" s="126">
         <f>MAX(AU20:AU23)-MIN(AU20:AU23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV24" s="126">
         <f>MAX(AV20:AV23)-MIN(AV20:AV23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW24" s="126">
         <f>MAX(AW20:AW23)-MIN(AW20:AW23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY24" s="126">
         <f>MAX(AY20:AY23)-MIN(AY20:AY23)+1</f>
@@ -45228,7 +45260,7 @@
       </c>
       <c r="AZ24" s="126">
         <f>MAX(AZ20:AZ23)+1</f>
-        <v>1</v>
+        <v>51.5</v>
       </c>
       <c r="BB24" s="126">
         <f>MAX(BB20:BB23)-MIN(BB20:BB23)+1</f>
@@ -45236,15 +45268,15 @@
       </c>
       <c r="BC24" s="126">
         <f>MAX(BC20:BC23)-MIN(BC20:BC23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BD24" s="126">
         <f>MAX(BD20:BD23)-MIN(BD20:BD23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BE24" s="126">
         <f>MAX(BE20:BE23)-MIN(BE20:BE23)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG24" s="126">
         <f>MAX(BG20:BG23)-MIN(BG20:BG23)+1</f>
@@ -45252,7 +45284,7 @@
       </c>
       <c r="BH24" s="126">
         <f>MAX(BH20:BH23)+1</f>
-        <v>1</v>
+        <v>51.5</v>
       </c>
       <c r="BL24" s="21"/>
       <c r="BM24" s="21"/>
@@ -45274,7 +45306,7 @@
       <c r="CC24" s="21"/>
       <c r="CD24" s="114"/>
       <c r="CE24" s="115"/>
-      <c r="CF24" s="164"/>
+      <c r="CF24" s="174"/>
       <c r="CG24" s="26" t="str">
         <f>IF(CD32&gt;CD33,BZ32,IF(CD32&lt;CD33,BZ33,""))</f>
         <v/>
@@ -45505,7 +45537,7 @@
       </c>
       <c r="AF26" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE26 &amp; "_win")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG26" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE26 &amp; "_draw")</f>
@@ -45517,31 +45549,31 @@
       </c>
       <c r="AI26" s="123">
         <f>SUMIF($E$7:$E$78,$AE26,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE26,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AJ26" s="123">
         <f>SUMIF($E$7:$E$78,$AE26,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE26,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL26" s="123">
         <f>AI26-AJ26</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AM26" s="123">
         <f>AL26-AL30</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN26" s="123">
         <f>AF26*3+AG26</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO26" s="123">
         <f>AN26/AN30*10+BA26</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="AP26" s="123">
         <f>AO26*10000000+BI26*100+AM26/AM30*10+AI26/AI30*1++IF(AQ26=0,ROW(),AQ26)/2000000</f>
-        <v>8.3656500000000005E-4</v>
+        <v>75000009.37226513</v>
       </c>
       <c r="AQ26" s="126">
         <f>VLOOKUP(AE26,db_fifarank,2,FALSE)</f>
@@ -45549,7 +45581,7 @@
       </c>
       <c r="AR26" s="125">
         <f>AP26/AP30</f>
-        <v>8.3586574397389256E-4</v>
+        <v>0.99999998666666856</v>
       </c>
       <c r="AS26" s="125" t="str">
         <f>IF(SUM(AF26:AH29)=12,J27,"1D")</f>
@@ -45619,7 +45651,7 @@
         <f>BH26/BH30</f>
         <v>0</v>
       </c>
-      <c r="BK26" s="163">
+      <c r="BK26" s="173">
         <v>83</v>
       </c>
       <c r="BL26" s="24" t="str">
@@ -45693,11 +45725,11 @@
       </c>
       <c r="K27" s="31">
         <f>L27+M27+N27</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="31">
         <f>VLOOKUP(1,AD26:AN29,3,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" s="31">
         <f>VLOOKUP(1,AD26:AN29,4,FALSE)</f>
@@ -45709,11 +45741,11 @@
       </c>
       <c r="O27" s="31" t="str">
         <f>VLOOKUP(1,AD26:AN29,6,FALSE) &amp; " - " &amp; VLOOKUP(1,AD26:AN29,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>4 - 1</v>
       </c>
       <c r="P27" s="32">
         <f>L27*3+M27</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R27" s="123">
         <f>DATE(2026,6,17)+TIME(12,0,0)+gmt_delta</f>
@@ -45777,19 +45809,19 @@
       </c>
       <c r="AH27" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE27 &amp; "_lose")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI27" s="123">
         <f>SUMIF($E$7:$E$78,$AE27,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE27,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ27" s="123">
         <f>SUMIF($E$7:$E$78,$AE27,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE27,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AL27" s="123">
         <f>AI27-AJ27</f>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="AM27" s="123">
         <f>AL27-AL30</f>
@@ -45805,7 +45837,7 @@
       </c>
       <c r="AP27" s="123">
         <f>AO27*10000000+BI27*100+AM27/AM30*10+AI27/AI30*1++IF(AQ27=0,ROW(),AQ27)/2000000</f>
-        <v>7.5175000000000003E-4</v>
+        <v>0.20075175000000001</v>
       </c>
       <c r="AQ27" s="126">
         <f>VLOOKUP(AE27,db_fifarank,2,FALSE)</f>
@@ -45813,7 +45845,7 @@
       </c>
       <c r="AR27" s="125">
         <f>AP27/AP30</f>
-        <v>7.5112163792696765E-4</v>
+        <v>2.6766896298222066E-9</v>
       </c>
       <c r="AS27" s="125" t="str">
         <f>IF(SUM(AF26:AH29)=12,J28,"2D")</f>
@@ -45883,7 +45915,7 @@
         <f>BH27/BH30</f>
         <v>0</v>
       </c>
-      <c r="BK27" s="164"/>
+      <c r="BK27" s="174"/>
       <c r="BL27" s="26" t="str">
         <f>AS75</f>
         <v>2L</v>
@@ -45957,15 +45989,15 @@
       </c>
       <c r="J28" s="33" t="str">
         <f>VLOOKUP(2,AD26:AN29,2,FALSE)</f>
-        <v>Turkey</v>
+        <v>Australia</v>
       </c>
       <c r="K28" s="23">
         <f>L28+M28+N28</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" s="23">
         <f>VLOOKUP(2,AD26:AN29,3,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M28" s="23">
         <f>VLOOKUP(2,AD26:AN29,4,FALSE)</f>
@@ -45977,11 +46009,11 @@
       </c>
       <c r="O28" s="23" t="str">
         <f>VLOOKUP(2,AD26:AN29,6,FALSE) &amp; " - " &amp; VLOOKUP(2,AD26:AN29,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>2 - 0</v>
       </c>
       <c r="P28" s="34">
         <f>L28*3+M28</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R28" s="123">
         <f>DATE(2026,6,17)+TIME(9,0,0)+gmt_delta</f>
@@ -46029,7 +46061,7 @@
       </c>
       <c r="AD28" s="123">
         <f>COUNTIF(AR26:AR29,CONCATENATE("&gt;=",AR28))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE28" s="124" t="str">
         <f>VLOOKUP("Australia",T,lang,FALSE)</f>
@@ -46037,7 +46069,7 @@
       </c>
       <c r="AF28" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE28 &amp; "_win")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG28" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE28 &amp; "_draw")</f>
@@ -46049,7 +46081,7 @@
       </c>
       <c r="AI28" s="123">
         <f>SUMIF($E$7:$E$78,$AE28,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE28,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ28" s="123">
         <f>SUMIF($E$7:$E$78,$AE28,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE28,$F$7:$F$78)</f>
@@ -46057,23 +46089,23 @@
       </c>
       <c r="AL28" s="123">
         <f>AI28-AJ28</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM28" s="123">
         <f>AL28-AL30</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AN28" s="123">
         <f>AF28*3+AG28</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO28" s="123">
         <f>AN28/AN30*10+BA28</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="AP28" s="123">
         <f>AO28*10000000+BI28*100+AM28/AM30*10+AI28/AI30*1++IF(AQ28=0,ROW(),AQ28)/2000000</f>
-        <v>7.9033500000000008E-4</v>
+        <v>75000007.543647483</v>
       </c>
       <c r="AQ28" s="126">
         <f>VLOOKUP(AE28,db_fifarank,2,FALSE)</f>
@@ -46081,7 +46113,7 @@
       </c>
       <c r="AR28" s="125">
         <f>AP28/AP30</f>
-        <v>7.8967438604723647E-4</v>
+        <v>0.99999996228510324</v>
       </c>
       <c r="AT28" s="126" cm="1">
         <f t="array" ref="AT28">SUMPRODUCT(($S$7:$S$78=AE28&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE28&amp;"_win")*($U$7:$U$78))</f>
@@ -46154,7 +46186,7 @@
       <c r="BO28" s="21"/>
       <c r="BP28" s="114"/>
       <c r="BQ28" s="112"/>
-      <c r="BR28" s="163">
+      <c r="BR28" s="173">
         <v>93</v>
       </c>
       <c r="BS28" s="24" t="str">
@@ -46212,11 +46244,11 @@
       </c>
       <c r="J29" s="33" t="str">
         <f>VLOOKUP(3,AD26:AN29,2,FALSE)</f>
-        <v>Australia</v>
+        <v>Turkey</v>
       </c>
       <c r="K29" s="23">
         <f>L29+M29+N29</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" s="23">
         <f>VLOOKUP(3,AD26:AN29,3,FALSE)</f>
@@ -46228,11 +46260,11 @@
       </c>
       <c r="N29" s="23">
         <f>VLOOKUP(3,AD26:AN29,5,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O29" s="23" t="str">
         <f>VLOOKUP(3,AD26:AN29,6,FALSE) &amp; " - " &amp; VLOOKUP(3,AD26:AN29,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>0 - 2</v>
       </c>
       <c r="P29" s="34">
         <f>L29*3+M29</f>
@@ -46284,7 +46316,7 @@
       </c>
       <c r="AD29" s="123">
         <f>COUNTIF(AR26:AR29,CONCATENATE("&gt;=",AR29))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE29" s="124" t="str">
         <f>VLOOKUP("Turkey",T,lang,FALSE)</f>
@@ -46300,7 +46332,7 @@
       </c>
       <c r="AH29" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE29 &amp; "_lose")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI29" s="123">
         <f>SUMIF($E$7:$E$78,$AE29,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE29,$G$7:$G$78)</f>
@@ -46308,15 +46340,15 @@
       </c>
       <c r="AJ29" s="123">
         <f>SUMIF($E$7:$E$78,$AE29,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE29,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AL29" s="123">
         <f>AI29-AJ29</f>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AM29" s="123">
         <f>AL29-AL30</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN29" s="123">
         <f>AF29*3+AG29</f>
@@ -46328,7 +46360,7 @@
       </c>
       <c r="AP29" s="123">
         <f>AO29*10000000+BI29*100+AM29/AM30*10+AI29/AI30*1++IF(AQ29=0,ROW(),AQ29)/2000000</f>
-        <v>7.9951999999999996E-4</v>
+        <v>1.4293709485714283</v>
       </c>
       <c r="AQ29" s="126">
         <f>VLOOKUP(AE29,db_fifarank,2,FALSE)</f>
@@ -46336,7 +46368,7 @@
       </c>
       <c r="AR29" s="125">
         <f>AP29/AP30</f>
-        <v>7.9885170862037803E-4</v>
+        <v>1.9058276678585728E-8</v>
       </c>
       <c r="AT29" s="126" cm="1">
         <f t="array" ref="AT29">SUMPRODUCT(($S$7:$S$78=AE29&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE29&amp;"_win")*($U$7:$U$78))</f>
@@ -46415,7 +46447,7 @@
         <v>46205.791666666672</v>
       </c>
       <c r="BQ29" s="115"/>
-      <c r="BR29" s="164"/>
+      <c r="BR29" s="174"/>
       <c r="BS29" s="26" t="str">
         <f>IF(BP30&gt;BP31,BL30,IF(BP30&lt;BP31,BL31,""))</f>
         <v/>
@@ -46475,7 +46507,7 @@
       </c>
       <c r="K30" s="36">
         <f>L30+M30+N30</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" s="36">
         <f>VLOOKUP(4,AD26:AN29,3,FALSE)</f>
@@ -46487,11 +46519,11 @@
       </c>
       <c r="N30" s="36">
         <f>VLOOKUP(4,AD26:AN29,5,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O30" s="36" t="str">
         <f>VLOOKUP(4,AD26:AN29,6,FALSE) &amp; " - " &amp; VLOOKUP(4,AD26:AN29,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 4</v>
       </c>
       <c r="P30" s="37">
         <f>L30*3+M30</f>
@@ -46543,7 +46575,7 @@
       </c>
       <c r="AF30" s="123">
         <f t="shared" ref="AF30:AH30" si="15">MAX(AF26:AF29)-MIN(AF26:AF29)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG30" s="123">
         <f t="shared" si="15"/>
@@ -46551,31 +46583,31 @@
       </c>
       <c r="AH30" s="123">
         <f t="shared" si="15"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI30" s="123">
         <f>MAX(AI26:AI29)+1</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AL30" s="123">
         <f>MIN(AL26:AL29)</f>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="AM30" s="123">
         <f>MAX(AM26:AM29)+1</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AN30" s="123">
         <f>MAX(AN26:AN29)+1</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AO30" s="123">
         <f>MAX(AO26:AO29)+1</f>
-        <v>1</v>
+        <v>8.5</v>
       </c>
       <c r="AP30" s="123">
         <f>MAX(AP26:AP29)+1</f>
-        <v>1.000836565</v>
+        <v>75000010.37226513</v>
       </c>
       <c r="AT30" s="126">
         <f>MAX(AT26:AT29)-MIN(AT26:AT29)+1</f>
@@ -46625,7 +46657,7 @@
         <f>MAX(BH26:BH29)+1</f>
         <v>1</v>
       </c>
-      <c r="BK30" s="163">
+      <c r="BK30" s="173">
         <v>84</v>
       </c>
       <c r="BL30" s="24" t="str">
@@ -46732,7 +46764,7 @@
         <f>IF(OR(F31="",G31=""),"",IF(F31&gt;G31,1,IF(F31&lt;G31,-1,0)))</f>
         <v/>
       </c>
-      <c r="BK31" s="164"/>
+      <c r="BK31" s="174"/>
       <c r="BL31" s="26" t="str">
         <f>AS63</f>
         <v>2J</v>
@@ -46876,7 +46908,7 @@
       </c>
       <c r="AF32" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE32 &amp; "_win")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG32" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE32 &amp; "_draw")</f>
@@ -46888,31 +46920,31 @@
       </c>
       <c r="AI32" s="123">
         <f>SUMIF($E$7:$E$78,$AE32,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE32,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AJ32" s="123">
         <f>SUMIF($E$7:$E$78,$AE32,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE32,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL32" s="123">
         <f>AI32-AJ32</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM32" s="123">
         <f>AL32-AL36</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="AN32" s="123">
         <f>AF32*3+AG32</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO32" s="123">
         <f>AN32/AN36*10+BA32</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="AP32" s="123">
         <f>AO32*10000000+BI32*100+AM32/AM36*10+AI32/AI36*1++IF(AQ32=0,ROW(),AQ32)/2000000</f>
-        <v>8.6518499999999998E-4</v>
+        <v>75000010.106634423</v>
       </c>
       <c r="AQ32" s="126">
         <f>VLOOKUP(AE32,db_fifarank,2,FALSE)</f>
@@ -46920,7 +46952,7 @@
       </c>
       <c r="AR32" s="125">
         <f>AP32/AP36</f>
-        <v>8.6443710198591821E-4</v>
+        <v>0.99999998666666867</v>
       </c>
       <c r="AS32" s="125" t="str">
         <f>IF(SUM(AF32:AH35)=12,J33,"1E")</f>
@@ -47004,7 +47036,7 @@
       <c r="BV32" s="21"/>
       <c r="BW32" s="114"/>
       <c r="BX32" s="112"/>
-      <c r="BY32" s="163">
+      <c r="BY32" s="173">
         <v>98</v>
       </c>
       <c r="BZ32" s="24" t="str">
@@ -47054,11 +47086,11 @@
       </c>
       <c r="K33" s="31">
         <f>L33+M33+N33</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="31">
         <f>VLOOKUP(1,AD32:AN35,3,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M33" s="31">
         <f>VLOOKUP(1,AD32:AN35,4,FALSE)</f>
@@ -47070,11 +47102,11 @@
       </c>
       <c r="O33" s="31" t="str">
         <f>VLOOKUP(1,AD32:AN35,6,FALSE) &amp; " - " &amp; VLOOKUP(1,AD32:AN35,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>7 - 1</v>
       </c>
       <c r="P33" s="32">
         <f>L33*3+M33</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R33" s="123">
         <f>DATE(2026,6,18)+TIME(11,0,0)+gmt_delta</f>
@@ -47138,19 +47170,19 @@
       </c>
       <c r="AH33" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE33 &amp; "_lose")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI33" s="123">
         <f>SUMIF($E$7:$E$78,$AE33,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE33,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ33" s="123">
         <f>SUMIF($E$7:$E$78,$AE33,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE33,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AL33" s="123">
         <f>AI33-AJ33</f>
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="AM33" s="123">
         <f>AL33-AL36</f>
@@ -47166,7 +47198,7 @@
       </c>
       <c r="AP33" s="123">
         <f>AO33*10000000+BI33*100+AM33/AM36*10+AI33/AI36*1++IF(AQ33=0,ROW(),AQ33)/2000000</f>
-        <v>6.4732500000000003E-4</v>
+        <v>0.125647325</v>
       </c>
       <c r="AQ33" s="126">
         <f>VLOOKUP(AE33,db_fifarank,2,FALSE)</f>
@@ -47174,7 +47206,7 @@
       </c>
       <c r="AR33" s="125">
         <f>AP33/AP36</f>
-        <v>6.4676542825295696E-4</v>
+        <v>1.6752974185744538E-9</v>
       </c>
       <c r="AS33" s="125" t="str">
         <f>IF(SUM(AF32:AH35)=12,J34,"2E")</f>
@@ -47264,7 +47296,7 @@
       <c r="BV33" s="21"/>
       <c r="BW33" s="114"/>
       <c r="BX33" s="115"/>
-      <c r="BY33" s="164"/>
+      <c r="BY33" s="174"/>
       <c r="BZ33" s="26" t="str">
         <f>IF(BW36&gt;BW37,BS36,IF(BW36&lt;BW37,BS37,""))</f>
         <v/>
@@ -47279,14 +47311,14 @@
       <c r="CE33" s="112"/>
       <c r="CK33" s="114"/>
       <c r="CL33" s="112"/>
-      <c r="CM33" s="165" t="str" cm="1">
+      <c r="CM33" s="176" t="str" cm="1">
         <f t="array" ref="CM33">INDEX(T,8,lang)</f>
         <v>Final</v>
       </c>
-      <c r="CN33" s="166"/>
-      <c r="CO33" s="166"/>
-      <c r="CP33" s="166"/>
-      <c r="CQ33" s="167"/>
+      <c r="CN33" s="177"/>
+      <c r="CO33" s="177"/>
+      <c r="CP33" s="177"/>
+      <c r="CQ33" s="178"/>
     </row>
     <row r="34" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A34" s="16">
@@ -47420,7 +47452,7 @@
       </c>
       <c r="AM34" s="123">
         <f>AL34-AL36</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN34" s="123">
         <f>AF34*3+AG34</f>
@@ -47432,7 +47464,7 @@
       </c>
       <c r="AP34" s="123">
         <f>AO34*10000000+BI34*100+AM34/AM36*10+AI34/AI36*1++IF(AQ34=0,ROW(),AQ34)/2000000</f>
-        <v>7.6648999999999999E-4</v>
+        <v>4.616151105384616</v>
       </c>
       <c r="AQ34" s="126">
         <f>VLOOKUP(AE34,db_fifarank,2,FALSE)</f>
@@ -47440,7 +47472,7 @@
       </c>
       <c r="AR34" s="125">
         <f>AP34/AP36</f>
-        <v>7.6582741760569868E-4</v>
+        <v>6.1548672290480187E-8</v>
       </c>
       <c r="AT34" s="126" cm="1">
         <f t="array" ref="AT34">SUMPRODUCT(($S$7:$S$78=AE34&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE34&amp;"_win")*($U$7:$U$78))</f>
@@ -47506,7 +47538,7 @@
         <f>BH34/BH36</f>
         <v>0</v>
       </c>
-      <c r="BK34" s="163">
+      <c r="BK34" s="173">
         <v>81</v>
       </c>
       <c r="BL34" s="24" t="str">
@@ -47537,11 +47569,11 @@
       <c r="CE34" s="112"/>
       <c r="CK34" s="114"/>
       <c r="CL34" s="112"/>
-      <c r="CM34" s="168"/>
-      <c r="CN34" s="169"/>
-      <c r="CO34" s="169"/>
-      <c r="CP34" s="169"/>
-      <c r="CQ34" s="170"/>
+      <c r="CM34" s="179"/>
+      <c r="CN34" s="180"/>
+      <c r="CO34" s="180"/>
+      <c r="CP34" s="180"/>
+      <c r="CQ34" s="181"/>
     </row>
     <row r="35" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A35" s="16">
@@ -47675,7 +47707,7 @@
       </c>
       <c r="AM35" s="123">
         <f>AL35-AL36</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN35" s="123">
         <f>AF35*3+AG35</f>
@@ -47687,7 +47719,7 @@
       </c>
       <c r="AP35" s="123">
         <f>AO35*10000000+BI35*100+AM35/AM36*10+AI35/AI36*1++IF(AQ35=0,ROW(),AQ35)/2000000</f>
-        <v>7.9739000000000003E-4</v>
+        <v>4.6161820053846156</v>
       </c>
       <c r="AQ35" s="126">
         <f>VLOOKUP(AE35,db_fifarank,2,FALSE)</f>
@@ -47695,7 +47727,7 @@
       </c>
       <c r="AR35" s="125">
         <f>AP35/AP36</f>
-        <v>7.9670070649924736E-4</v>
+        <v>6.154908429041916E-8</v>
       </c>
       <c r="AT35" s="126" cm="1">
         <f t="array" ref="AT35">SUMPRODUCT(($S$7:$S$78=AE35&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE35&amp;"_win")*($U$7:$U$78))</f>
@@ -47761,7 +47793,7 @@
         <f>BH35/BH36</f>
         <v>0</v>
       </c>
-      <c r="BK35" s="164"/>
+      <c r="BK35" s="174"/>
       <c r="BL35" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!F3,AK80:AS91,9,FALSE),"3rd Group B/E/F/I/J")</f>
         <v>3rd Group B/E/F/I/J</v>
@@ -47829,7 +47861,7 @@
       </c>
       <c r="K36" s="36">
         <f>L36+M36+N36</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" s="36">
         <f>VLOOKUP(4,AD32:AN35,3,FALSE)</f>
@@ -47841,11 +47873,11 @@
       </c>
       <c r="N36" s="36">
         <f>VLOOKUP(4,AD32:AN35,5,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O36" s="36" t="str">
         <f>VLOOKUP(4,AD32:AN35,6,FALSE) &amp; " - " &amp; VLOOKUP(4,AD32:AN35,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 7</v>
       </c>
       <c r="P36" s="37">
         <f>L36*3+M36</f>
@@ -47897,7 +47929,7 @@
       </c>
       <c r="AF36" s="123">
         <f t="shared" ref="AF36:AH36" si="16">MAX(AF32:AF35)-MIN(AF32:AF35)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG36" s="123">
         <f t="shared" si="16"/>
@@ -47905,31 +47937,31 @@
       </c>
       <c r="AH36" s="123">
         <f t="shared" si="16"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI36" s="123">
         <f>MAX(AI32:AI35)+1</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AL36" s="123">
         <f>MIN(AL32:AL35)</f>
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="AM36" s="123">
         <f>MAX(AM32:AM35)+1</f>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="AN36" s="123">
         <f>MAX(AN32:AN35)+1</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AO36" s="123">
         <f>MAX(AO32:AO35)+1</f>
-        <v>1</v>
+        <v>8.5</v>
       </c>
       <c r="AP36" s="123">
         <f>MAX(AP32:AP35)+1</f>
-        <v>1.0008651850000001</v>
+        <v>75000011.106634423</v>
       </c>
       <c r="AT36" s="126">
         <f>MAX(AT32:AT35)-MIN(AT32:AT35)+1</f>
@@ -47986,7 +48018,7 @@
       <c r="BO36" s="21"/>
       <c r="BP36" s="114"/>
       <c r="BQ36" s="112"/>
-      <c r="BR36" s="163">
+      <c r="BR36" s="173">
         <v>94</v>
       </c>
       <c r="BS36" s="24" t="str">
@@ -48106,7 +48138,7 @@
         <v>46204.833333333336</v>
       </c>
       <c r="BQ37" s="115"/>
-      <c r="BR37" s="164"/>
+      <c r="BR37" s="174"/>
       <c r="BS37" s="26" t="str">
         <f>IF(BP38&gt;BP39,BL38,IF(BP38&lt;BP39,BL39,""))</f>
         <v/>
@@ -48133,7 +48165,7 @@
       <c r="CJ37" s="21"/>
       <c r="CK37" s="114"/>
       <c r="CL37" s="112"/>
-      <c r="CM37" s="163">
+      <c r="CM37" s="173">
         <v>104</v>
       </c>
       <c r="CN37" s="24" t="str">
@@ -48260,7 +48292,7 @@
       </c>
       <c r="AG38" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE38 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH38" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE38 &amp; "_lose")</f>
@@ -48268,11 +48300,11 @@
       </c>
       <c r="AI38" s="123">
         <f>SUMIF($E$7:$E$78,$AE38,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE38,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ38" s="123">
         <f>SUMIF($E$7:$E$78,$AE38,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE38,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AL38" s="123">
         <f>AI38-AJ38</f>
@@ -48284,15 +48316,15 @@
       </c>
       <c r="AN38" s="123">
         <f>AF38*3+AG38</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO38" s="123">
         <f>AN38/AN42*10+BA38</f>
-        <v>0</v>
+        <v>5.9806451612903224</v>
       </c>
       <c r="AP38" s="123">
         <f>AO38*10000000+BI38*100+AM38/AM42*10+AI38/AI42*1++IF(AQ38=0,ROW(),AQ38)/2000000</f>
-        <v>8.7893499999999996E-4</v>
+        <v>59806550.344964951</v>
       </c>
       <c r="AQ38" s="126">
         <f>VLOOKUP(AE38,db_fifarank,2,FALSE)</f>
@@ -48300,7 +48332,7 @@
       </c>
       <c r="AR38" s="125">
         <f>AP38/AP42</f>
-        <v>8.7816315167028663E-4</v>
+        <v>0.99999998327942374</v>
       </c>
       <c r="AS38" s="125" t="str">
         <f>IF(SUM(AF38:AH41)=12,J39,"1F")</f>
@@ -48312,15 +48344,15 @@
       </c>
       <c r="AU38" s="126" cm="1">
         <f t="array" ref="AU38">SUMPRODUCT(($S$7:$S$78=AE38&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE38&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV38" s="126" cm="1">
         <f t="array" ref="AV38">SUMPRODUCT(($E$7:$E$78=AE38)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE38)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW38" s="126" cm="1">
         <f t="array" ref="AW38">SUMPRODUCT(($E$7:$E$78=AE38)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE38)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AX38" s="126">
         <f>AV38-AW38</f>
@@ -48332,11 +48364,11 @@
       </c>
       <c r="AZ38" s="126">
         <f>AT38/AT42*1000+AU38/AU42*100+AY38/AY42*10+AV38/AV42</f>
-        <v>0</v>
+        <v>50.666666666666664</v>
       </c>
       <c r="BA38" s="126">
         <f>AZ38/AZ42</f>
-        <v>0</v>
+        <v>0.98064516129032253</v>
       </c>
       <c r="BB38" s="126" cm="1">
         <f t="array" ref="BB38">SUMPRODUCT(($S$7:$S$78=AE38&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE38&amp;"_win")*($X$7:$X$78))</f>
@@ -48344,15 +48376,15 @@
       </c>
       <c r="BC38" s="126" cm="1">
         <f t="array" ref="BC38">SUMPRODUCT(($S$7:$S$78=AE38&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE38&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD38" s="126" cm="1">
         <f t="array" ref="BD38">SUMPRODUCT(($E$7:$E$78=AE38)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE38)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BE38" s="126" cm="1">
         <f t="array" ref="BE38">SUMPRODUCT(($E$7:$E$78=AE38)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE38)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BF38" s="126">
         <f>BD38-BE38</f>
@@ -48364,13 +48396,13 @@
       </c>
       <c r="BH38" s="126">
         <f>BB38/BB42*1000+BC38/BC42*100+BG38/BG42*10+BD38/BD42</f>
-        <v>0</v>
+        <v>50.666666666666664</v>
       </c>
       <c r="BI38" s="126">
         <f>BH38/BH42</f>
-        <v>0</v>
-      </c>
-      <c r="BK38" s="163">
+        <v>0.98064516129032253</v>
+      </c>
+      <c r="BK38" s="173">
         <v>82</v>
       </c>
       <c r="BL38" s="24" t="str">
@@ -48400,7 +48432,7 @@
       <c r="CI38" s="21"/>
       <c r="CJ38" s="21"/>
       <c r="CL38" s="115"/>
-      <c r="CM38" s="164"/>
+      <c r="CM38" s="174"/>
       <c r="CN38" s="26" t="str">
         <f>IF(CK55&gt;CK56,CG55,IF(CK55&lt;CK56,CG56,""))</f>
         <v/>
@@ -48445,7 +48477,7 @@
       </c>
       <c r="K39" s="31">
         <f>L39+M39+N39</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" s="31">
         <f>VLOOKUP(1,AD38:AN41,3,FALSE)</f>
@@ -48453,7 +48485,7 @@
       </c>
       <c r="M39" s="31">
         <f>VLOOKUP(1,AD38:AN41,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N39" s="31">
         <f>VLOOKUP(1,AD38:AN41,5,FALSE)</f>
@@ -48461,11 +48493,11 @@
       </c>
       <c r="O39" s="31" t="str">
         <f>VLOOKUP(1,AD38:AN41,6,FALSE) &amp; " - " &amp; VLOOKUP(1,AD38:AN41,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>2 - 2</v>
       </c>
       <c r="P39" s="32">
         <f>L39*3+M39</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R39" s="123">
         <f>DATE(2026,6,20)+TIME(9,0,0)+gmt_delta</f>
@@ -48525,7 +48557,7 @@
       </c>
       <c r="AG39" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE39 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH39" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE39 &amp; "_lose")</f>
@@ -48533,11 +48565,11 @@
       </c>
       <c r="AI39" s="123">
         <f>SUMIF($E$7:$E$78,$AE39,$F$7:$F$78) + SUMIF($H$7:$H$78,$AE39,$G$7:$G$78)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ39" s="123">
         <f>SUMIF($E$7:$E$78,$AE39,$G$7:$G$78) + SUMIF($H$7:$H$78,$AE39,$F$7:$F$78)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AL39" s="123">
         <f>AI39-AJ39</f>
@@ -48549,15 +48581,15 @@
       </c>
       <c r="AN39" s="123">
         <f>AF39*3+AG39</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO39" s="123">
         <f>AN39/AN42*10+BA39</f>
-        <v>0</v>
+        <v>5.9806451612903224</v>
       </c>
       <c r="AP39" s="123">
         <f>AO39*10000000+BI39*100+AM39/AM42*10+AI39/AI42*1++IF(AQ39=0,ROW(),AQ39)/2000000</f>
-        <v>8.3021500000000003E-4</v>
+        <v>59806550.344916232</v>
       </c>
       <c r="AQ39" s="126">
         <f>VLOOKUP(AE39,db_fifarank,2,FALSE)</f>
@@ -48565,7 +48597,7 @@
       </c>
       <c r="AR39" s="125">
         <f>AP39/AP42</f>
-        <v>8.2948593577903611E-4</v>
+        <v>0.99999998327860917</v>
       </c>
       <c r="AS39" s="125" t="str">
         <f>IF(SUM(AF38:AH41)=12,J40,"2F")</f>
@@ -48577,15 +48609,15 @@
       </c>
       <c r="AU39" s="126" cm="1">
         <f t="array" ref="AU39">SUMPRODUCT(($S$7:$S$78=AE39&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE39&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV39" s="126" cm="1">
         <f t="array" ref="AV39">SUMPRODUCT(($E$7:$E$78=AE39)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE39)*($U$7:$U$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW39" s="126" cm="1">
         <f t="array" ref="AW39">SUMPRODUCT(($E$7:$E$78=AE39)*($U$7:$U$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE39)*($U$7:$U$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AX39" s="126">
         <f>AV39-AW39</f>
@@ -48597,11 +48629,11 @@
       </c>
       <c r="AZ39" s="126">
         <f>AT39/AT42*1000+AU39/AU42*100+AY39/AY42*10+AV39/AV42</f>
-        <v>0</v>
+        <v>50.666666666666664</v>
       </c>
       <c r="BA39" s="126">
         <f>AZ39/AZ42</f>
-        <v>0</v>
+        <v>0.98064516129032253</v>
       </c>
       <c r="BB39" s="126" cm="1">
         <f t="array" ref="BB39">SUMPRODUCT(($S$7:$S$78=AE39&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE39&amp;"_win")*($X$7:$X$78))</f>
@@ -48609,15 +48641,15 @@
       </c>
       <c r="BC39" s="126" cm="1">
         <f t="array" ref="BC39">SUMPRODUCT(($S$7:$S$78=AE39&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE39&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD39" s="126" cm="1">
         <f t="array" ref="BD39">SUMPRODUCT(($E$7:$E$78=AE39)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE39)*($X$7:$X$78)*($G$7:$G$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BE39" s="126" cm="1">
         <f t="array" ref="BE39">SUMPRODUCT(($E$7:$E$78=AE39)*($X$7:$X$78)*($G$7:$G$78))+SUMPRODUCT(($H$7:$H$78=AE39)*($X$7:$X$78)*($F$7:$F$78))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BF39" s="126">
         <f>BD39-BE39</f>
@@ -48629,13 +48661,13 @@
       </c>
       <c r="BH39" s="126">
         <f>BB39/BB42*1000+BC39/BC42*100+BG39/BG42*10+BD39/BD42</f>
-        <v>0</v>
+        <v>50.666666666666664</v>
       </c>
       <c r="BI39" s="126">
         <f>BH39/BH42</f>
-        <v>0</v>
-      </c>
-      <c r="BK39" s="164"/>
+        <v>0.98064516129032253</v>
+      </c>
+      <c r="BK39" s="174"/>
       <c r="BL39" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!H3,AK80:AS91,9,FALSE),"3rd Group A/E/H/I/J")</f>
         <v>3rd Group A/E/H/I/J</v>
@@ -48700,7 +48732,7 @@
       </c>
       <c r="K40" s="23">
         <f>L40+M40+N40</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" s="23">
         <f>VLOOKUP(2,AD38:AN41,3,FALSE)</f>
@@ -48708,7 +48740,7 @@
       </c>
       <c r="M40" s="23">
         <f>VLOOKUP(2,AD38:AN41,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N40" s="23">
         <f>VLOOKUP(2,AD38:AN41,5,FALSE)</f>
@@ -48716,11 +48748,11 @@
       </c>
       <c r="O40" s="23" t="str">
         <f>VLOOKUP(2,AD38:AN41,6,FALSE) &amp; " - " &amp; VLOOKUP(2,AD38:AN41,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>2 - 2</v>
       </c>
       <c r="P40" s="34">
         <f>L40*3+M40</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R40" s="123">
         <f>DATE(2026,6,20)+TIME(13,0,0)+gmt_delta</f>
@@ -48820,7 +48852,7 @@
       </c>
       <c r="AR40" s="125">
         <f>AP40/AP42</f>
-        <v>7.5671989240137219E-4</v>
+        <v>1.2663913617613456E-11</v>
       </c>
       <c r="AT40" s="126" cm="1">
         <f t="array" ref="AT40">SUMPRODUCT(($S$7:$S$78=AE40&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE40&amp;"_win")*($U$7:$U$78))</f>
@@ -49041,7 +49073,7 @@
       </c>
       <c r="AR41" s="125">
         <f>AP41/AP42</f>
-        <v>7.4087382006895759E-4</v>
+        <v>1.2398725278822286E-11</v>
       </c>
       <c r="AT41" s="126" cm="1">
         <f t="array" ref="AT41">SUMPRODUCT(($S$7:$S$78=AE41&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE41&amp;"_win")*($U$7:$U$78))</f>
@@ -49233,7 +49265,7 @@
       </c>
       <c r="AG42" s="123">
         <f t="shared" si="18"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH42" s="123">
         <f t="shared" si="18"/>
@@ -49241,7 +49273,7 @@
       </c>
       <c r="AI42" s="123">
         <f>MAX(AI38:AI41)+1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AL42" s="123">
         <f>MIN(AL38:AL41)</f>
@@ -49253,15 +49285,15 @@
       </c>
       <c r="AN42" s="123">
         <f>MAX(AN38:AN41)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO42" s="123">
         <f>MAX(AO38:AO41)+1</f>
-        <v>1</v>
+        <v>6.9806451612903224</v>
       </c>
       <c r="AP42" s="123">
         <f>MAX(AP38:AP41)+1</f>
-        <v>1.000878935</v>
+        <v>59806551.344964951</v>
       </c>
       <c r="AT42" s="126">
         <f>MAX(AT38:AT41)-MIN(AT38:AT41)+1</f>
@@ -49269,15 +49301,15 @@
       </c>
       <c r="AU42" s="126">
         <f>MAX(AU38:AU41)-MIN(AU38:AU41)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV42" s="126">
         <f>MAX(AV38:AV41)-MIN(AV38:AV41)+1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW42" s="126">
         <f>MAX(AW38:AW41)-MIN(AW38:AW41)+1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AY42" s="126">
         <f>MAX(AY38:AY41)-MIN(AY38:AY41)+1</f>
@@ -49285,7 +49317,7 @@
       </c>
       <c r="AZ42" s="126">
         <f>MAX(AZ38:AZ41)+1</f>
-        <v>1</v>
+        <v>51.666666666666664</v>
       </c>
       <c r="BB42" s="126">
         <f>MAX(BB38:BB41)-MIN(BB38:BB41)+1</f>
@@ -49293,15 +49325,15 @@
       </c>
       <c r="BC42" s="126">
         <f>MAX(BC38:BC41)-MIN(BC38:BC41)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BD42" s="126">
         <f>MAX(BD38:BD41)-MIN(BD38:BD41)+1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BE42" s="126">
         <f>MAX(BE38:BE41)-MIN(BE38:BE41)+1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG42" s="126">
         <f>MAX(BG38:BG41)-MIN(BG38:BG41)+1</f>
@@ -49309,9 +49341,9 @@
       </c>
       <c r="BH42" s="126">
         <f>MAX(BH38:BH41)+1</f>
-        <v>1</v>
-      </c>
-      <c r="BK42" s="163">
+        <v>51.666666666666664</v>
+      </c>
+      <c r="BK42" s="173">
         <v>76</v>
       </c>
       <c r="BL42" s="24" t="str">
@@ -49404,7 +49436,7 @@
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="BK43" s="164"/>
+      <c r="BK43" s="174"/>
       <c r="BL43" s="26" t="str">
         <f>AS39</f>
         <v>2F</v>
@@ -49660,7 +49692,7 @@
       <c r="BO44" s="21"/>
       <c r="BP44" s="114"/>
       <c r="BQ44" s="112"/>
-      <c r="BR44" s="163">
+      <c r="BR44" s="173">
         <v>91</v>
       </c>
       <c r="BS44" s="24" t="str">
@@ -49675,14 +49707,14 @@
         <v/>
       </c>
       <c r="CK44" s="114"/>
-      <c r="CM44" s="165" t="str" cm="1">
+      <c r="CM44" s="176" t="str" cm="1">
         <f t="array" ref="CM44">INDEX(T,7,lang)</f>
         <v>Third-Place Play-Off</v>
       </c>
-      <c r="CN44" s="166"/>
-      <c r="CO44" s="166"/>
-      <c r="CP44" s="166"/>
-      <c r="CQ44" s="167"/>
+      <c r="CN44" s="177"/>
+      <c r="CO44" s="177"/>
+      <c r="CP44" s="177"/>
+      <c r="CQ44" s="178"/>
     </row>
     <row r="45" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="16">
@@ -49919,7 +49951,7 @@
         <v>46203.708333333336</v>
       </c>
       <c r="BQ45" s="115"/>
-      <c r="BR45" s="164"/>
+      <c r="BR45" s="174"/>
       <c r="BS45" s="26" t="str">
         <f>IF(BP46&gt;BP47,BL46,IF(BP46&lt;BP47,BL47,""))</f>
         <v/>
@@ -49932,11 +49964,11 @@
         <v/>
       </c>
       <c r="CK45" s="114"/>
-      <c r="CM45" s="168"/>
-      <c r="CN45" s="169"/>
-      <c r="CO45" s="169"/>
-      <c r="CP45" s="169"/>
-      <c r="CQ45" s="170"/>
+      <c r="CM45" s="179"/>
+      <c r="CN45" s="180"/>
+      <c r="CO45" s="180"/>
+      <c r="CP45" s="180"/>
+      <c r="CQ45" s="181"/>
     </row>
     <row r="46" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A46" s="16">
@@ -50156,7 +50188,7 @@
         <f>BH46/BH48</f>
         <v>0</v>
       </c>
-      <c r="BK46" s="163">
+      <c r="BK46" s="173">
         <v>78</v>
       </c>
       <c r="BL46" s="24" t="str">
@@ -50398,7 +50430,7 @@
         <f>BH47/BH48</f>
         <v>0</v>
       </c>
-      <c r="BK47" s="164"/>
+      <c r="BK47" s="174"/>
       <c r="BL47" s="26" t="str">
         <f>AS57</f>
         <v>2I</v>
@@ -50641,7 +50673,7 @@
       <c r="BV48" s="21"/>
       <c r="BW48" s="114"/>
       <c r="BX48" s="112"/>
-      <c r="BY48" s="163">
+      <c r="BY48" s="173">
         <v>99</v>
       </c>
       <c r="BZ48" s="24" t="str">
@@ -50657,7 +50689,7 @@
       </c>
       <c r="CK48" s="114"/>
       <c r="CL48" s="112"/>
-      <c r="CM48" s="163">
+      <c r="CM48" s="173">
         <v>103</v>
       </c>
       <c r="CN48" s="24" t="str">
@@ -50762,7 +50794,7 @@
       <c r="BV49" s="21"/>
       <c r="BW49" s="114"/>
       <c r="BX49" s="115"/>
-      <c r="BY49" s="164"/>
+      <c r="BY49" s="174"/>
       <c r="BZ49" s="26" t="str">
         <f>IF(BW52&gt;BW53,BS52,IF(BW52&lt;BW53,BS53,""))</f>
         <v/>
@@ -50776,7 +50808,7 @@
       </c>
       <c r="CK49" s="114"/>
       <c r="CL49" s="115"/>
-      <c r="CM49" s="164"/>
+      <c r="CM49" s="174"/>
       <c r="CN49" s="26" t="str">
         <f>IF(CK55&gt;CK56,CG56,IF(CK55&lt;CK56,CG55,""))</f>
         <v/>
@@ -51011,7 +51043,7 @@
         <f>BH50/BH54</f>
         <v>0</v>
       </c>
-      <c r="BK50" s="163">
+      <c r="BK50" s="173">
         <v>79</v>
       </c>
       <c r="BL50" s="24" t="str">
@@ -51264,7 +51296,7 @@
         <f>BH51/BH54</f>
         <v>0</v>
       </c>
-      <c r="BK51" s="164"/>
+      <c r="BK51" s="174"/>
       <c r="BL51" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!D3,AK80:AS91,9,FALSE),"3rd Group C/E/F/H/I")</f>
         <v>3rd Group C/E/F/H/I</v>
@@ -51524,7 +51556,7 @@
       <c r="BO52" s="21"/>
       <c r="BP52" s="114"/>
       <c r="BQ52" s="112"/>
-      <c r="BR52" s="163">
+      <c r="BR52" s="173">
         <v>92</v>
       </c>
       <c r="BS52" s="24" t="str">
@@ -51779,7 +51811,7 @@
         <v>46204.666666666672</v>
       </c>
       <c r="BQ53" s="115"/>
-      <c r="BR53" s="164"/>
+      <c r="BR53" s="174"/>
       <c r="BS53" s="26" t="str">
         <f>IF(BP54&gt;BP55,BL54,IF(BP54&lt;BP55,BL55,""))</f>
         <v/>
@@ -51983,7 +52015,7 @@
         <f>MAX(BH50:BH53)+1</f>
         <v>1</v>
       </c>
-      <c r="BK54" s="163">
+      <c r="BK54" s="173">
         <v>80</v>
       </c>
       <c r="BL54" s="24" t="str">
@@ -52104,7 +52136,7 @@
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="BK55" s="164"/>
+      <c r="BK55" s="174"/>
       <c r="BL55" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!K3,AK80:AS91,9,FALSE),"3rd Group E/H/I/J/K")</f>
         <v>3rd Group E/H/I/J/K</v>
@@ -52131,7 +52163,7 @@
       <c r="CC55" s="21"/>
       <c r="CD55" s="114"/>
       <c r="CE55" s="112"/>
-      <c r="CF55" s="163">
+      <c r="CF55" s="173">
         <v>102</v>
       </c>
       <c r="CG55" s="24" t="str">
@@ -52390,7 +52422,7 @@
       <c r="CC56" s="21"/>
       <c r="CD56" s="114"/>
       <c r="CE56" s="115"/>
-      <c r="CF56" s="164"/>
+      <c r="CF56" s="174"/>
       <c r="CG56" s="26" t="str">
         <f>IF(CD64&gt;CD65,BZ64,IF(CD64&lt;CD65,BZ65,""))</f>
         <v/>
@@ -52873,7 +52905,7 @@
         <f>BH58/BH60</f>
         <v>0</v>
       </c>
-      <c r="BK58" s="163">
+      <c r="BK58" s="173">
         <v>86</v>
       </c>
       <c r="BL58" s="24" t="str">
@@ -53121,7 +53153,7 @@
         <f>BH59/BH60</f>
         <v>0</v>
       </c>
-      <c r="BK59" s="164"/>
+      <c r="BK59" s="174"/>
       <c r="BL59" s="26" t="str">
         <f>AS51</f>
         <v>2H</v>
@@ -53344,7 +53376,7 @@
       <c r="BO60" s="21"/>
       <c r="BP60" s="114"/>
       <c r="BQ60" s="112"/>
-      <c r="BR60" s="163">
+      <c r="BR60" s="173">
         <v>95</v>
       </c>
       <c r="BS60" s="24" t="str">
@@ -53457,7 +53489,7 @@
         <v>46206.75</v>
       </c>
       <c r="BQ61" s="115"/>
-      <c r="BR61" s="164"/>
+      <c r="BR61" s="174"/>
       <c r="BS61" s="26" t="str">
         <f>IF(BP62&gt;BP63,BL62,IF(BP62&lt;BP63,BL63,""))</f>
         <v/>
@@ -53700,7 +53732,7 @@
         <f>BH62/BH66</f>
         <v>0</v>
       </c>
-      <c r="BK62" s="163">
+      <c r="BK62" s="173">
         <v>88</v>
       </c>
       <c r="BL62" s="24" t="str">
@@ -53952,7 +53984,7 @@
         <f>BH63/BH66</f>
         <v>0</v>
       </c>
-      <c r="BK63" s="164"/>
+      <c r="BK63" s="174"/>
       <c r="BL63" s="26" t="str">
         <f>AS45</f>
         <v>2G</v>
@@ -54218,7 +54250,7 @@
       <c r="BV64" s="21"/>
       <c r="BW64" s="114"/>
       <c r="BX64" s="112"/>
-      <c r="BY64" s="163">
+      <c r="BY64" s="173">
         <v>100</v>
       </c>
       <c r="BZ64" s="24" t="str">
@@ -54472,7 +54504,7 @@
       <c r="BV65" s="21"/>
       <c r="BW65" s="114"/>
       <c r="BX65" s="115"/>
-      <c r="BY65" s="164"/>
+      <c r="BY65" s="174"/>
       <c r="BZ65" s="26" t="str">
         <f>IF(BW68&gt;BW69,BS68,IF(BW68&lt;BW69,BS69,""))</f>
         <v/>
@@ -54668,7 +54700,7 @@
         <f>MAX(BH62:BH65)+1</f>
         <v>1</v>
       </c>
-      <c r="BK66" s="163">
+      <c r="BK66" s="173">
         <v>85</v>
       </c>
       <c r="BL66" s="24" t="str">
@@ -54768,7 +54800,7 @@
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="BK67" s="164"/>
+      <c r="BK67" s="174"/>
       <c r="BL67" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!E3,AK80:AS91,9,FALSE),"3rd Group E/F/G/I/J")</f>
         <v>3rd Group E/F/G/I/J</v>
@@ -55024,7 +55056,7 @@
       <c r="BO68" s="21"/>
       <c r="BP68" s="114"/>
       <c r="BQ68" s="112"/>
-      <c r="BR68" s="163">
+      <c r="BR68" s="173">
         <v>96</v>
       </c>
       <c r="BS68" s="24" t="str">
@@ -55038,25 +55070,25 @@
         <f>IF(OR(BT68="",BT69="",AND(BU68="",BU69&lt;&gt;""),AND(BU69="",BU68&lt;&gt;""),AND(BV68="",BV69&lt;&gt;""),AND(BV69="",BV68&lt;&gt;"")),"",BT68*1000+BU68*10+BV68)</f>
         <v/>
       </c>
-      <c r="CE68" s="195" t="str">
+      <c r="CE68" s="175" t="str">
         <f>INDEX(T,144,lang)</f>
         <v>World Champion 2026</v>
       </c>
-      <c r="CF68" s="195"/>
-      <c r="CG68" s="195"/>
-      <c r="CH68" s="195"/>
-      <c r="CI68" s="195"/>
-      <c r="CJ68" s="195"/>
-      <c r="CK68" s="185" t="str">
+      <c r="CF68" s="175"/>
+      <c r="CG68" s="175"/>
+      <c r="CH68" s="175"/>
+      <c r="CI68" s="175"/>
+      <c r="CJ68" s="175"/>
+      <c r="CK68" s="163" t="str">
         <f>IF(CR37&gt;CR38,CN37,IF(CR37&lt;CR38,CN38,""))</f>
         <v/>
       </c>
-      <c r="CL68" s="185"/>
-      <c r="CM68" s="185"/>
-      <c r="CN68" s="185"/>
-      <c r="CO68" s="185"/>
-      <c r="CP68" s="185"/>
-      <c r="CQ68" s="185"/>
+      <c r="CL68" s="163"/>
+      <c r="CM68" s="163"/>
+      <c r="CN68" s="163"/>
+      <c r="CO68" s="163"/>
+      <c r="CP68" s="163"/>
+      <c r="CQ68" s="163"/>
     </row>
     <row r="69" spans="1:95" x14ac:dyDescent="0.2">
       <c r="A69" s="16">
@@ -55294,7 +55326,7 @@
         <v>46207.0625</v>
       </c>
       <c r="BQ69" s="115"/>
-      <c r="BR69" s="164"/>
+      <c r="BR69" s="174"/>
       <c r="BS69" s="26" t="str">
         <f>IF(BP70&gt;BP71,BL70,IF(BP70&lt;BP71,BL71,""))</f>
         <v/>
@@ -55306,19 +55338,19 @@
         <f>IF(BW68="","",BT69*1000+BU69*10+BV69)</f>
         <v/>
       </c>
-      <c r="CE69" s="195"/>
-      <c r="CF69" s="195"/>
-      <c r="CG69" s="195"/>
-      <c r="CH69" s="195"/>
-      <c r="CI69" s="195"/>
-      <c r="CJ69" s="195"/>
-      <c r="CK69" s="185"/>
-      <c r="CL69" s="185"/>
-      <c r="CM69" s="185"/>
-      <c r="CN69" s="185"/>
-      <c r="CO69" s="185"/>
-      <c r="CP69" s="185"/>
-      <c r="CQ69" s="185"/>
+      <c r="CE69" s="175"/>
+      <c r="CF69" s="175"/>
+      <c r="CG69" s="175"/>
+      <c r="CH69" s="175"/>
+      <c r="CI69" s="175"/>
+      <c r="CJ69" s="175"/>
+      <c r="CK69" s="163"/>
+      <c r="CL69" s="163"/>
+      <c r="CM69" s="163"/>
+      <c r="CN69" s="163"/>
+      <c r="CO69" s="163"/>
+      <c r="CP69" s="163"/>
+      <c r="CQ69" s="163"/>
     </row>
     <row r="70" spans="1:95" x14ac:dyDescent="0.2">
       <c r="A70" s="16">
@@ -55539,7 +55571,7 @@
         <f>BH70/BH72</f>
         <v>0</v>
       </c>
-      <c r="BK70" s="163">
+      <c r="BK70" s="173">
         <v>87</v>
       </c>
       <c r="BL70" s="24" t="str">
@@ -55775,7 +55807,7 @@
         <f>BH71/BH72</f>
         <v>0</v>
       </c>
-      <c r="BK71" s="164"/>
+      <c r="BK71" s="174"/>
       <c r="BL71" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!J3,AK80:AS91,9,FALSE),"3rd Group D/E/I/J/L")</f>
         <v>3rd Group D/E/I/J/L</v>
@@ -57182,7 +57214,7 @@
       </c>
       <c r="AD80" s="123">
         <f>COUNTIF($AP$80:$AP$91,CONCATENATE("&gt;=",AP80))</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AE80" s="124" t="str">
         <f>J11</f>
@@ -57217,7 +57249,7 @@
       </c>
       <c r="AM80" s="123">
         <f>AL80-$AL$92</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN80" s="123">
         <f>VLOOKUP($AE80,$AE$8:$AQ$78,10,FALSE)</f>
@@ -57225,7 +57257,7 @@
       </c>
       <c r="AP80" s="123">
         <f>AN80/AN92*10000+AM80/AM92*1000+AI80/AI92*100+IF(AQ80=0,ROW(),AQ80)/2000000</f>
-        <v>50.000750689999997</v>
+        <v>383.33408402333333</v>
       </c>
       <c r="AQ80" s="126">
         <f t="shared" ref="AQ80:AQ91" si="37">VLOOKUP($AE80,$AE$8:$AQ$78,13,FALSE)</f>
@@ -57256,11 +57288,11 @@
       <c r="I81" s="69"/>
       <c r="J81" s="96" t="str">
         <f>VLOOKUP(1,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓓ Australia</v>
+        <v>Ⓒ Morocco</v>
       </c>
       <c r="K81" s="97">
         <f>L81+M81+N81</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L81" s="97">
         <f>VLOOKUP(1,$AD$80:$AN$91,3,FALSE)</f>
@@ -57268,7 +57300,7 @@
       </c>
       <c r="M81" s="97">
         <f>VLOOKUP(1,$AD$80:$AN$91,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N81" s="97">
         <f>VLOOKUP(1,$AD$80:$AN$91,5,FALSE)</f>
@@ -57276,15 +57308,15 @@
       </c>
       <c r="O81" s="97" t="str">
         <f>VLOOKUP(1,$AD$80:$AN$91,6,FALSE) &amp; " - " &amp; VLOOKUP(1,$AD$80:$AN$91,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P81" s="98">
         <f>L81*3+M81</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD81" s="123">
         <f t="shared" ref="AD81:AD91" si="38">COUNTIF($AP$80:$AP$91,CONCATENATE("&gt;=",AP81))</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AE81" s="124" t="str">
         <f>J17</f>
@@ -57296,7 +57328,7 @@
       </c>
       <c r="AG81" s="123">
         <f>VLOOKUP($AE81,$AE$8:$AQ$78,3,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH81" s="123">
         <f t="shared" ref="AH81:AH90" si="40">VLOOKUP($AE81,$AE$8:$AQ$78,4,FALSE)</f>
@@ -57304,11 +57336,11 @@
       </c>
       <c r="AI81" s="123">
         <f t="shared" ref="AI81:AI90" si="41">VLOOKUP($AE81,$AE$8:$AQ$78,5,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ81" s="123">
         <f t="shared" ref="AJ81:AJ90" si="42">VLOOKUP($AE81,$AE$8:$AQ$78,6,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK81" s="123" t="s">
         <v>3181</v>
@@ -57319,15 +57351,15 @@
       </c>
       <c r="AM81" s="123">
         <f t="shared" ref="AM81:AM91" si="44">AL81-$AL$92</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN81" s="123">
         <f t="shared" ref="AN81:AN90" si="45">VLOOKUP($AE81,$AE$8:$AQ$78,10,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP81" s="123">
         <f>AN81/AN92*10000+AM81/AM92*1000+AI81/AI92*100+IF(AQ81=0,ROW(),AQ81)/2000000</f>
-        <v>500.00072748000002</v>
+        <v>5716.667394146667</v>
       </c>
       <c r="AQ81" s="126">
         <f t="shared" si="37"/>
@@ -57335,11 +57367,11 @@
       </c>
       <c r="AR81" s="125" t="str">
         <f>AR80&amp;IF(AD81&lt;=8,RIGHT(AK81,1),"")</f>
-        <v/>
+        <v>B</v>
       </c>
       <c r="AS81" s="129" t="str">
         <f t="shared" ref="AS81:AS91" si="46">IF(AD81&lt;=8,AE81,"")</f>
-        <v/>
+        <v>Qatar</v>
       </c>
       <c r="AT81" s="130" t="str">
         <f>"Ⓑ "&amp;AE81</f>
@@ -57358,11 +57390,11 @@
       <c r="I82" s="69"/>
       <c r="J82" s="99" t="str">
         <f>VLOOKUP(2,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓙ Algeria</v>
+        <v>Ⓑ Qatar</v>
       </c>
       <c r="K82" s="100">
         <f t="shared" ref="K82:K92" si="47">L82+M82+N82</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" s="100">
         <f>VLOOKUP(2,$AD$80:$AN$91,3,FALSE)</f>
@@ -57370,7 +57402,7 @@
       </c>
       <c r="M82" s="100">
         <f>VLOOKUP(2,$AD$80:$AN$91,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N82" s="100">
         <f>VLOOKUP(2,$AD$80:$AN$91,5,FALSE)</f>
@@ -57378,19 +57410,19 @@
       </c>
       <c r="O82" s="100" t="str">
         <f>VLOOKUP(2,$AD$80:$AN$91,6,FALSE) &amp; " - " &amp; VLOOKUP(2,$AD$80:$AN$91,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 1</v>
       </c>
       <c r="P82" s="101">
         <f t="shared" ref="P82:P92" si="48">L82*3+M82</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD82" s="123">
         <f t="shared" si="38"/>
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AE82" s="124" t="str">
         <f>J23</f>
-        <v>Scotland</v>
+        <v>Morocco</v>
       </c>
       <c r="AF82" s="123">
         <f t="shared" si="39"/>
@@ -57398,7 +57430,7 @@
       </c>
       <c r="AG82" s="123">
         <f t="shared" ref="AG82:AG91" si="49">VLOOKUP($AE82,$AE$8:$AQ$78,3,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH82" s="123">
         <f t="shared" si="40"/>
@@ -57406,11 +57438,11 @@
       </c>
       <c r="AI82" s="123">
         <f t="shared" si="41"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ82" s="123">
         <f t="shared" si="42"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK82" s="123" t="s">
         <v>3182</v>
@@ -57421,48 +57453,48 @@
       </c>
       <c r="AM82" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN82" s="123">
         <f t="shared" si="45"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP82" s="123">
         <f>AN82/AN92*10000+AM82/AM92*1000+AI82/AI92*100+IF(AQ82=0,ROW(),AQ82)/2000000</f>
-        <v>500.00074917500001</v>
+        <v>5716.667544601667</v>
       </c>
       <c r="AQ82" s="126">
         <f t="shared" si="37"/>
-        <v>1498.35</v>
+        <v>1755.87</v>
       </c>
       <c r="AR82" s="125" t="str">
         <f t="shared" ref="AR82:AR91" si="50">AR81&amp;IF(AD82&lt;=8,RIGHT(AK82,1),"")</f>
-        <v>C</v>
+        <v>BC</v>
       </c>
       <c r="AS82" s="129" t="str">
         <f t="shared" si="46"/>
-        <v>Scotland</v>
+        <v>Morocco</v>
       </c>
       <c r="AT82" s="130" t="str">
         <f>"Ⓒ "&amp;AE82</f>
-        <v>Ⓒ Scotland</v>
+        <v>Ⓒ Morocco</v>
       </c>
     </row>
     <row r="83" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="73"/>
       <c r="B83" s="73"/>
-      <c r="C83" s="186" t="s">
+      <c r="C83" s="164" t="s">
         <v>3183</v>
       </c>
-      <c r="D83" s="187"/>
-      <c r="E83" s="187"/>
-      <c r="F83" s="187"/>
-      <c r="G83" s="188"/>
+      <c r="D83" s="165"/>
+      <c r="E83" s="165"/>
+      <c r="F83" s="165"/>
+      <c r="G83" s="166"/>
       <c r="H83" s="75"/>
       <c r="I83" s="69"/>
       <c r="J83" s="99" t="str">
         <f>VLOOKUP(3,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓖ Egypt</v>
+        <v>Ⓙ Algeria</v>
       </c>
       <c r="K83" s="100">
         <f t="shared" si="47"/>
@@ -57490,11 +57522,11 @@
       </c>
       <c r="AD83" s="123">
         <f t="shared" si="38"/>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="AE83" s="124" t="str">
         <f>J29</f>
-        <v>Australia</v>
+        <v>Turkey</v>
       </c>
       <c r="AF83" s="123">
         <f t="shared" si="39"/>
@@ -57506,7 +57538,7 @@
       </c>
       <c r="AH83" s="123">
         <f t="shared" si="40"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI83" s="123">
         <f t="shared" si="41"/>
@@ -57514,18 +57546,18 @@
       </c>
       <c r="AJ83" s="123">
         <f t="shared" si="42"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AK83" s="123" t="s">
         <v>3184</v>
       </c>
       <c r="AL83" s="123">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AM83" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN83" s="123">
         <f t="shared" si="45"/>
@@ -57533,38 +57565,38 @@
       </c>
       <c r="AP83" s="123">
         <f>AN83/AN92*10000+AM83/AM92*1000+AI83/AI92*100+IF(AQ83=0,ROW(),AQ83)/2000000</f>
-        <v>500.00079033499998</v>
+        <v>7.9951999999999996E-4</v>
       </c>
       <c r="AQ83" s="126">
         <f t="shared" si="37"/>
-        <v>1580.67</v>
+        <v>1599.04</v>
       </c>
       <c r="AR83" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CD</v>
+        <v>BC</v>
       </c>
       <c r="AS83" s="129" t="str">
         <f t="shared" si="46"/>
-        <v>Australia</v>
+        <v/>
       </c>
       <c r="AT83" s="130" t="str">
         <f>"Ⓓ "&amp;AE83</f>
-        <v>Ⓓ Australia</v>
+        <v>Ⓓ Turkey</v>
       </c>
     </row>
     <row r="84" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="73"/>
       <c r="B84" s="73"/>
-      <c r="C84" s="189"/>
-      <c r="D84" s="190"/>
-      <c r="E84" s="190"/>
-      <c r="F84" s="190"/>
-      <c r="G84" s="191"/>
+      <c r="C84" s="167"/>
+      <c r="D84" s="168"/>
+      <c r="E84" s="168"/>
+      <c r="F84" s="168"/>
+      <c r="G84" s="169"/>
       <c r="H84" s="75"/>
       <c r="I84" s="69"/>
       <c r="J84" s="99" t="str">
         <f>VLOOKUP(4,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓘ Norway</v>
+        <v>Ⓖ Egypt</v>
       </c>
       <c r="K84" s="100">
         <f t="shared" si="47"/>
@@ -57604,7 +57636,7 @@
       </c>
       <c r="AD84" s="123">
         <f t="shared" si="38"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE84" s="124" t="str">
         <f>J35</f>
@@ -57639,7 +57671,7 @@
       </c>
       <c r="AM84" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN84" s="123">
         <f t="shared" si="45"/>
@@ -57647,7 +57679,7 @@
       </c>
       <c r="AP84" s="123">
         <f>AN84/AN92*10000+AM84/AM92*1000+AI84/AI92*100+IF(AQ84=0,ROW(),AQ84)/2000000</f>
-        <v>500.00076648999999</v>
+        <v>666.66743315666668</v>
       </c>
       <c r="AQ84" s="126">
         <f t="shared" si="37"/>
@@ -57655,7 +57687,7 @@
       </c>
       <c r="AR84" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDE</v>
+        <v>BCE</v>
       </c>
       <c r="AS84" s="129" t="str">
         <f t="shared" si="46"/>
@@ -57669,16 +57701,16 @@
     <row r="85" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="73"/>
       <c r="B85" s="73"/>
-      <c r="C85" s="189"/>
-      <c r="D85" s="190"/>
-      <c r="E85" s="190"/>
-      <c r="F85" s="190"/>
-      <c r="G85" s="191"/>
+      <c r="C85" s="167"/>
+      <c r="D85" s="168"/>
+      <c r="E85" s="168"/>
+      <c r="F85" s="168"/>
+      <c r="G85" s="169"/>
       <c r="H85" s="75"/>
       <c r="I85" s="69"/>
       <c r="J85" s="99" t="str">
         <f>VLOOKUP(5,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓛ Panama</v>
+        <v>Ⓘ Norway</v>
       </c>
       <c r="K85" s="100">
         <f t="shared" si="47"/>
@@ -57718,7 +57750,7 @@
       </c>
       <c r="AD85" s="123">
         <f t="shared" si="38"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AE85" s="124" t="str">
         <f>J41</f>
@@ -57753,7 +57785,7 @@
       </c>
       <c r="AM85" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN85" s="123">
         <f t="shared" si="45"/>
@@ -57761,7 +57793,7 @@
       </c>
       <c r="AP85" s="123">
         <f>AN85/AN92*10000+AM85/AM92*1000+AI85/AI92*100+IF(AQ85=0,ROW(),AQ85)/2000000</f>
-        <v>500.00075738499999</v>
+        <v>666.66742405166667</v>
       </c>
       <c r="AQ85" s="126">
         <f t="shared" si="37"/>
@@ -57769,7 +57801,7 @@
       </c>
       <c r="AR85" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDEF</v>
+        <v>BCEF</v>
       </c>
       <c r="AS85" s="129" t="str">
         <f t="shared" si="46"/>
@@ -57783,16 +57815,16 @@
     <row r="86" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="73"/>
       <c r="B86" s="73"/>
-      <c r="C86" s="189"/>
-      <c r="D86" s="190"/>
-      <c r="E86" s="190"/>
-      <c r="F86" s="190"/>
-      <c r="G86" s="191"/>
+      <c r="C86" s="167"/>
+      <c r="D86" s="168"/>
+      <c r="E86" s="168"/>
+      <c r="F86" s="168"/>
+      <c r="G86" s="169"/>
       <c r="H86" s="75"/>
       <c r="I86" s="69"/>
       <c r="J86" s="99" t="str">
         <f>VLOOKUP(6,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓔ Ivory Coast</v>
+        <v>Ⓛ Panama</v>
       </c>
       <c r="K86" s="100">
         <f t="shared" si="47"/>
@@ -57832,7 +57864,7 @@
       </c>
       <c r="AD86" s="123">
         <f t="shared" si="38"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE86" s="124" t="str">
         <f>J47</f>
@@ -57867,7 +57899,7 @@
       </c>
       <c r="AM86" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN86" s="123">
         <f t="shared" si="45"/>
@@ -57875,7 +57907,7 @@
       </c>
       <c r="AP86" s="123">
         <f>AN86/AN92*10000+AM86/AM92*1000+AI86/AI92*100+IF(AQ86=0,ROW(),AQ86)/2000000</f>
-        <v>500.00078162</v>
+        <v>666.66744828666663</v>
       </c>
       <c r="AQ86" s="126">
         <f t="shared" si="37"/>
@@ -57883,7 +57915,7 @@
       </c>
       <c r="AR86" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDEFG</v>
+        <v>BCEFG</v>
       </c>
       <c r="AS86" s="129" t="str">
         <f t="shared" si="46"/>
@@ -57897,16 +57929,16 @@
     <row r="87" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="73"/>
       <c r="B87" s="73"/>
-      <c r="C87" s="189"/>
-      <c r="D87" s="190"/>
-      <c r="E87" s="190"/>
-      <c r="F87" s="190"/>
-      <c r="G87" s="191"/>
+      <c r="C87" s="167"/>
+      <c r="D87" s="168"/>
+      <c r="E87" s="168"/>
+      <c r="F87" s="168"/>
+      <c r="G87" s="169"/>
       <c r="H87" s="75"/>
       <c r="I87" s="69"/>
       <c r="J87" s="99" t="str">
         <f>VLOOKUP(7,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓕ Sweden</v>
+        <v>Ⓔ Ivory Coast</v>
       </c>
       <c r="K87" s="100">
         <f t="shared" si="47"/>
@@ -57946,7 +57978,7 @@
       </c>
       <c r="AD87" s="123">
         <f t="shared" si="38"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AE87" s="124" t="str">
         <f>J53</f>
@@ -57981,7 +58013,7 @@
       </c>
       <c r="AM87" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN87" s="123">
         <f t="shared" si="45"/>
@@ -57989,7 +58021,7 @@
       </c>
       <c r="AP87" s="123">
         <f>AN87/AN92*10000+AM87/AM92*1000+AI87/AI92*100+IF(AQ87=0,ROW(),AQ87)/2000000</f>
-        <v>500.00071071500003</v>
+        <v>666.6673773816666</v>
       </c>
       <c r="AQ87" s="126">
         <f t="shared" si="37"/>
@@ -57997,7 +58029,7 @@
       </c>
       <c r="AR87" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDEFG</v>
+        <v>BCEFG</v>
       </c>
       <c r="AS87" s="129" t="str">
         <f t="shared" si="46"/>
@@ -58011,16 +58043,16 @@
     <row r="88" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="73"/>
       <c r="B88" s="73"/>
-      <c r="C88" s="192"/>
-      <c r="D88" s="193"/>
-      <c r="E88" s="193"/>
-      <c r="F88" s="193"/>
-      <c r="G88" s="194"/>
+      <c r="C88" s="170"/>
+      <c r="D88" s="171"/>
+      <c r="E88" s="171"/>
+      <c r="F88" s="171"/>
+      <c r="G88" s="172"/>
       <c r="H88" s="75"/>
       <c r="I88" s="69"/>
       <c r="J88" s="99" t="str">
         <f>VLOOKUP(8,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓒ Scotland</v>
+        <v>Ⓕ Sweden</v>
       </c>
       <c r="K88" s="100">
         <f t="shared" si="47"/>
@@ -58060,7 +58092,7 @@
       </c>
       <c r="AD88" s="123">
         <f t="shared" si="38"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AE88" s="124" t="str">
         <f>J59</f>
@@ -58095,7 +58127,7 @@
       </c>
       <c r="AM88" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN88" s="123">
         <f t="shared" si="45"/>
@@ -58103,7 +58135,7 @@
       </c>
       <c r="AP88" s="123">
         <f>AN88/AN92*10000+AM88/AM92*1000+AI88/AI92*100+IF(AQ88=0,ROW(),AQ88)/2000000</f>
-        <v>500.00077547000001</v>
+        <v>666.66744213666664</v>
       </c>
       <c r="AQ88" s="126">
         <f t="shared" si="37"/>
@@ -58111,7 +58143,7 @@
       </c>
       <c r="AR88" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDEFGI</v>
+        <v>BCEFGI</v>
       </c>
       <c r="AS88" s="129" t="str">
         <f t="shared" si="46"/>
@@ -58174,7 +58206,7 @@
       </c>
       <c r="AD89" s="123">
         <f t="shared" si="38"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE89" s="124" t="str">
         <f>J65</f>
@@ -58209,7 +58241,7 @@
       </c>
       <c r="AM89" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN89" s="123">
         <f t="shared" si="45"/>
@@ -58217,7 +58249,7 @@
       </c>
       <c r="AP89" s="123">
         <f>AN89/AN92*10000+AM89/AM92*1000+AI89/AI92*100+IF(AQ89=0,ROW(),AQ89)/2000000</f>
-        <v>500.00078213</v>
+        <v>666.66744879666658</v>
       </c>
       <c r="AQ89" s="126">
         <f t="shared" si="37"/>
@@ -58225,7 +58257,7 @@
       </c>
       <c r="AR89" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDEFGIJ</v>
+        <v>BCEFGIJ</v>
       </c>
       <c r="AS89" s="129" t="str">
         <f t="shared" si="46"/>
@@ -58248,7 +58280,7 @@
       <c r="I90" s="69"/>
       <c r="J90" s="102" t="str">
         <f>VLOOKUP(10,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓑ Qatar</v>
+        <v>Ⓗ Saudi Arabia</v>
       </c>
       <c r="K90" s="103">
         <f t="shared" si="47"/>
@@ -58323,7 +58355,7 @@
       </c>
       <c r="AM90" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN90" s="123">
         <f t="shared" si="45"/>
@@ -58331,7 +58363,7 @@
       </c>
       <c r="AP90" s="123">
         <f>AN90/AN92*10000+AM90/AM92*1000+AI90/AI92*100+IF(AQ90=0,ROW(),AQ90)/2000000</f>
-        <v>500.00073917499998</v>
+        <v>666.66740584166666</v>
       </c>
       <c r="AQ90" s="126">
         <f t="shared" si="37"/>
@@ -58339,7 +58371,7 @@
       </c>
       <c r="AR90" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDEFGIJ</v>
+        <v>BCEFGIJ</v>
       </c>
       <c r="AS90" s="129" t="str">
         <f t="shared" si="46"/>
@@ -58362,11 +58394,11 @@
       <c r="I91" s="69"/>
       <c r="J91" s="102" t="str">
         <f>VLOOKUP(11,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓗ Saudi Arabia</v>
+        <v>Ⓐ Czech Republic</v>
       </c>
       <c r="K91" s="103">
         <f t="shared" si="47"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L91" s="103">
         <f>VLOOKUP(11,$AD$80:$AN$91,3,FALSE)</f>
@@ -58378,11 +58410,11 @@
       </c>
       <c r="N91" s="103">
         <f>VLOOKUP(11,$AD$80:$AN$91,5,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O91" s="103" t="str">
         <f>VLOOKUP(11,$AD$80:$AN$91,6,FALSE) &amp; " - " &amp; VLOOKUP(11,$AD$80:$AN$91,7,FALSE)</f>
-        <v>0 - 0</v>
+        <v>1 - 2</v>
       </c>
       <c r="P91" s="104">
         <f t="shared" si="48"/>
@@ -58402,7 +58434,7 @@
       </c>
       <c r="AD91" s="123">
         <f t="shared" si="38"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE91" s="124" t="str">
         <f>J77</f>
@@ -58437,7 +58469,7 @@
       </c>
       <c r="AM91" s="123">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN91" s="123">
         <f>VLOOKUP($AE91,$AE$8:$AQ$78,10,FALSE)</f>
@@ -58445,7 +58477,7 @@
       </c>
       <c r="AP91" s="123">
         <f>AN91/AN92*10000+AM91/AM92*1000+AI91/AI92*100+IF(AQ91=0,ROW(),AQ91)/2000000</f>
-        <v>500.00077032000002</v>
+        <v>666.66743698666664</v>
       </c>
       <c r="AQ91" s="126">
         <f t="shared" si="37"/>
@@ -58453,7 +58485,7 @@
       </c>
       <c r="AR91" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>CDEFGIJL</v>
+        <v>BCEFGIJL</v>
       </c>
       <c r="AS91" s="129" t="str">
         <f t="shared" si="46"/>
@@ -58476,7 +58508,7 @@
       <c r="I92" s="69"/>
       <c r="J92" s="105" t="str">
         <f>VLOOKUP(12,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓐ Czech Republic</v>
+        <v>Ⓓ Turkey</v>
       </c>
       <c r="K92" s="106">
         <f t="shared" si="47"/>
@@ -58496,7 +58528,7 @@
       </c>
       <c r="O92" s="106" t="str">
         <f>VLOOKUP(12,$AD$80:$AN$91,6,FALSE) &amp; " - " &amp; VLOOKUP(12,$AD$80:$AN$91,7,FALSE)</f>
-        <v>1 - 2</v>
+        <v>0 - 2</v>
       </c>
       <c r="P92" s="107">
         <f t="shared" si="48"/>
@@ -58508,7 +58540,7 @@
       </c>
       <c r="AG92" s="123">
         <f>MAX(AG80:AG91)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH92" s="123">
         <f>MAX(AH80:AH91)+1</f>
@@ -58524,15 +58556,15 @@
       </c>
       <c r="AL92" s="123">
         <f>MIN(AL80:AL91)</f>
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AM92" s="123">
         <f>MAX(AM80:AM91)+1</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN92" s="123">
         <f>MAX(AN80:AN91)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS92" s="126" t="b">
         <f>SUM(K9:K78)=144</f>
@@ -58693,6 +58725,36 @@
   <sheetProtection algorithmName="SHA-512" hashValue="7nWuIQAsd0NKRlhwUK3tOeNHpTch5B5FULy2gxNNaIdJM5RfhFSMzPcx55y+pmM3d73guUy+p5Y+SvIjJZQRaA==" saltValue="Uw23KnM8csnTioq5H8upCA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <dataConsolidate/>
   <mergeCells count="45">
+    <mergeCell ref="BK14:BK15"/>
+    <mergeCell ref="BY16:BY17"/>
+    <mergeCell ref="BK26:BK27"/>
+    <mergeCell ref="BR28:BR29"/>
+    <mergeCell ref="BK22:BK23"/>
+    <mergeCell ref="CF23:CF24"/>
+    <mergeCell ref="BK18:BK19"/>
+    <mergeCell ref="BR20:BR21"/>
+    <mergeCell ref="CM48:CM49"/>
+    <mergeCell ref="BR44:BR45"/>
+    <mergeCell ref="BK46:BK47"/>
+    <mergeCell ref="BK30:BK31"/>
+    <mergeCell ref="CM44:CQ45"/>
+    <mergeCell ref="BY32:BY33"/>
+    <mergeCell ref="BK38:BK39"/>
+    <mergeCell ref="BK34:BK35"/>
+    <mergeCell ref="BR36:BR37"/>
+    <mergeCell ref="BK42:BK43"/>
+    <mergeCell ref="CM33:CQ34"/>
+    <mergeCell ref="CM37:CM38"/>
+    <mergeCell ref="BK10:BK11"/>
+    <mergeCell ref="BR12:BR13"/>
+    <mergeCell ref="BK6:BO7"/>
+    <mergeCell ref="BR6:BV7"/>
+    <mergeCell ref="BY6:CC7"/>
+    <mergeCell ref="CF6:CJ7"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="A5:H6"/>
+    <mergeCell ref="J5:P6"/>
     <mergeCell ref="CK68:CQ69"/>
     <mergeCell ref="C83:G88"/>
     <mergeCell ref="BK70:BK71"/>
@@ -58708,36 +58770,6 @@
     <mergeCell ref="BR52:BR53"/>
     <mergeCell ref="BK54:BK55"/>
     <mergeCell ref="CE68:CJ69"/>
-    <mergeCell ref="CF6:CJ7"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="A5:H6"/>
-    <mergeCell ref="J5:P6"/>
-    <mergeCell ref="BK10:BK11"/>
-    <mergeCell ref="BR12:BR13"/>
-    <mergeCell ref="BK6:BO7"/>
-    <mergeCell ref="BR6:BV7"/>
-    <mergeCell ref="BY6:CC7"/>
-    <mergeCell ref="CF23:CF24"/>
-    <mergeCell ref="BK18:BK19"/>
-    <mergeCell ref="BR20:BR21"/>
-    <mergeCell ref="CM48:CM49"/>
-    <mergeCell ref="BR44:BR45"/>
-    <mergeCell ref="BK46:BK47"/>
-    <mergeCell ref="BK30:BK31"/>
-    <mergeCell ref="CM44:CQ45"/>
-    <mergeCell ref="BY32:BY33"/>
-    <mergeCell ref="BK38:BK39"/>
-    <mergeCell ref="BK34:BK35"/>
-    <mergeCell ref="BR36:BR37"/>
-    <mergeCell ref="BK42:BK43"/>
-    <mergeCell ref="CM33:CQ34"/>
-    <mergeCell ref="CM37:CM38"/>
-    <mergeCell ref="BK14:BK15"/>
-    <mergeCell ref="BY16:BY17"/>
-    <mergeCell ref="BK26:BK27"/>
-    <mergeCell ref="BR28:BR29"/>
-    <mergeCell ref="BK22:BK23"/>
   </mergeCells>
   <conditionalFormatting sqref="A7:E78">
     <cfRule type="expression" dxfId="228" priority="339">
@@ -60034,15 +60066,15 @@
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B3" s="109">
         <f>MATCH(C3,C6:C500,0)</f>
-        <v>38</v>
+        <v>102</v>
       </c>
       <c r="C3" s="121" t="str">
         <f>'2026 World Cup'!AR91</f>
-        <v>CDEFGIJL</v>
+        <v>BCEFGIJL</v>
       </c>
       <c r="D3" s="121" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,2,FALSE)</f>
-        <v>3C</v>
+        <v>3E</v>
       </c>
       <c r="E3" s="121" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,3,FALSE)</f>
@@ -60050,11 +60082,11 @@
       </c>
       <c r="F3" s="121" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,4,FALSE)</f>
-        <v>3E</v>
+        <v>3B</v>
       </c>
       <c r="G3" s="121" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,5,FALSE)</f>
-        <v>3D</v>
+        <v>3C</v>
       </c>
       <c r="H3" s="121" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,6,FALSE)</f>

</xml_diff>